<commit_message>
test: record security review and pilot evidence (SEC-01, SYS-03, PRF-01)
Bandit review and secrets check rows, SYS-03 isolation/revocation/
offline evidence and PRF-01 budgets from the Stage 5F pilot record (pilot
limits L1 and L2 logged as DEF-11 and DEF-10), TC-06/TC-07 not executed
(second PC not available), TC-15 awaiting the Product Owner, and the
latest Testing Kanban sync logs.
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Owner'!$A$1:$G$10</definedName>
@@ -54,17 +54,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -549,136 +549,144 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 10:45</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.3</t>
+          <t>PRF-01.P1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 940e082 / 9e18f30</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>pip install -r requirements-dev.txt succeeds.</t>
+          <t>Pilot budget: p95 upload acknowledgement (pending -&gt; synced, online) &lt;= 5 s.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Exit code 0. Every requirement was already satisfied; nothing changed.</t>
+          <t>PC A: '1.33-2.09 s across 5 runs; manual 1.22 s'. PC B: '2.08-4.46 s across 6 runs; 24.06 s on live capture 6 (2026-10-10)'. Pilot verdict: 'Not met on one run. Met on the other 11, including the 2026-10-16 live retest (3.44 s). Limit L2'.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>DEF-10</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/pip-install-requirements-dev.log; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4, §5 finding 3, §7 L2; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 10:45</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.4</t>
+          <t>PRF-01.P2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 940e082 / 9e18f30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>pip install pytest-cov pip-audit bandit succeeds.</t>
+          <t>Pilot budget: sustained acknowledged events per client &gt;= 20 events/s.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Exit code 0. Installed pytest-cov 7.1.0 and coverage 7.16.2; pip-audit 2.10.1 and bandit 1.9.4 were already installed.</t>
+          <t>PC A: '≈ 1.9/s (capture 5: 300 events in 157 s)'. PC B: 'backlog drain of 210 events in 4.1 s ≈ 51/s'. Pilot verdict: 'Not demonstrated. Sources are paced by design: CSV Fast emits one flow per 0.35 s, ≤ 2.9/s. Each capture stores at most 300 events. Limit L1'.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/pip-install-test-tools.log; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4, §5 finding 4, §7 L1; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 10:45</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.7</t>
+          <t>PRF-01.P4</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 940e082</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bundled datasets present and row counts recorded; UNSW_NB15_training-set.csv has 82,332 rows.</t>
+          <t>Pilot budget: live capture packet drop &lt;= 1%.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>datasets/algoguard_big.csv 5,000 rows (1,597 Normal / 3,403 Attack); algoguard_bigger.csv 10,000 (3,194 / 6,806); algoguard_biggest.csv 20,000 (6,388 / 13,612); research/dataset/raw/UNSW_NB15_training-set.csv 82,332 rows, 45 columns (37,000 Normal / 45,332 Attack). SHA-256 of each file recorded.</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
+          <t>PC A: '0% (0 of 848; 0 of 2,810)'. PC B: '0% (0 of 119,100; 0 of 740)'. Pilot verdict: 'Met'.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -686,47 +694,47 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/dataset_counts.json; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 10:46</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.8</t>
+          <t>PRF-01.P5</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 9e18f30</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Independent evaluation set built from the UNSW-NB15 training set with every row seen in training removed; row counts recorded (plan 5.1).</t>
+          <t>Pilot budget: AlgoGuard process CPU peak &lt;= 50% of the machine.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>82,332 rows loaded; 29,089 removed because their 15 features match a row in datasets/*.csv; 53,243 kept (20,674 Attack / 32,569 Normal). Generic attacks fall from 18,871 to 802 rows after removal; 7,387 kept rows repeat the features of another kept row.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
+          <t>PC A: '24.5% (2-s samples, Test C)'. PC B: '6.3% (2-s samples, capture 18)'. Pilot verdict: 'Met'. Not the plan 3.4 soak budget (&lt;= 80% over 30 min).</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -734,24 +742,24 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/independent_set_counts.json (built with scripts/evaluate_model.py row_keys()); evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 10:51</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>TC-16</t>
+          <t>PRF-01.P6</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ENV-02</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -761,20 +769,20 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 9e18f30</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Line coverage of services/ &gt;= 80% (pytest --cov=services).</t>
+          <t>Pilot budget: AlgoGuard process RAM (working set) peak &lt;= 1 GB.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>TOTAL 1,869 statements, 312 missed: 83% line coverage. 537 passed, 67 deselected (integration lane), 18 warnings (all ResourceWarning: unclosed sqlite3 connection, from test_live_monitor and test_model_architecture) in 290.45 s. Below 80% per module: traffic_source_service 69%, deployment_service 77%.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
+          <t>PC A: '294 MB'. PC B: '108 MB'. Pilot verdict: 'Met'. PC A samples cover 07:58-08:43Z on 2026-10-08 (first 32 min of a 46-min CSV run); PC B's cover 60 s of capture 18.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -782,95 +790,95 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>test-results/coverage_20261019_104655/pytest-cov.log; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:00</t>
+          <t>2026-10-08 to 2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.9</t>
+          <t>PRF-01.P7</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 940e082 / 9e18f30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Official UNSW_NB15_testing-set.csv (175,341 rows) in research/dataset/raw/ for model B (SYS-01).</t>
+          <t>Pilot budget: local state-folder growth per PC, whole pilot &lt;= 50 MB.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Not executed: the file is not on this PC (checked 10:45 and 13:00). An alternative for the model B comparison is to be decided at Checkpoint 1.</t>
+          <t>PC A: '0.051 -&gt; 8.846 MiB (8.162 MiB is the model)'. PC B: '9.12 MiB in total'. Pilot verdict: 'Met'.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Not executed</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/dataset_counts.json; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:00</t>
+          <t>2026-10-16 (pilot)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.10</t>
+          <t>PRF-01.P3</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 9e18f30 (PC B)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Second PC for the two-PC pilot confirmed, or reported unavailable to the Test Lead (ENV-01 card).</t>
+          <t>Pilot budget: average live event-to-verdict lag &lt;= 20 s (measured from a flow's last packet, so it includes the 15 s idle timeout).</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>PC B is not available on 2026-10-19. Reported in this log and in the Test Status Report (DOC-05). Plan section 8 contingency applies: SYS-03 hardware steps Not executed; the automated two-node integration tests (INT-01) cover isolation.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
+          <t>PC A: 'not recorded'. PC B: '13.1 s' (capture 19, 2026-10-16). Pilot verdict: 'Met on PC B; not recorded on PC A'. This is not the plan 3.4 budget (p95 &lt;= 500 ms excluding timeouts), which TC-11 measures.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -878,151 +886,143 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Lead Architect's answer, 2026-10-19 13:00; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §2, §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:00</t>
+          <t>2026-10-16 (pilot; time not stated)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ENV-02.1</t>
+          <t>SYS-03.P1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>ENV-02</t>
+          <t>SYS-03</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Cel Hendrix N. San Miguel</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 4c9666c / 940e082</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
+          <t>Each node only sees its own data; no record crosses nodes (SYS-03 card).</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>CI workflow (windows-latest) failed on cb3bcdb (run 38886300881, 2026-10-16) and on 940e082 (runs 38870178965 on 2026-10-16 and 38017196080 on 2026-10-10). In both 2026-10-16 runs: Lint success, Type check success, Unit tests failure ('Process completed with exit code 1'), Browser polling tests skipped. All six runs listed for main (back to 4c9666c, 2026-10-05) concluded failure.</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>DEF-01</t>
-        </is>
-      </c>
+          <t>Pilot record: 'The two node UUIDs differ and each persisted across every restart from 2026-10-08 to 2026-10-16, including the deliberate restart in Test E.' (PC A d535e2fd-8392-4876-a945-c8d9c5184049, PC B 265f767e-f540-4f71-bf36-c7364f99ba59). 'No row was written under the other client's node or owner. Analysts can read only their own node, and the Administrator can read both.'</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>GitHub REST API (unauthenticated) actions/runs and jobs for main; job logs need sign-in (HTTP 403); evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §1 (Accounts and nodes) and §7 (accepted on the physical pilot); 2026-10-08 to 2026-10-16; Tests A-D on 4c9666c, 2026-10-15/16 work on 940e082</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:03</t>
+          <t>2026-10-16 (pilot; time not stated)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ENV-02.2</t>
+          <t>SYS-03.P2</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ENV-02</t>
+          <t>SYS-03</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Cel Hendrix N. San Miguel</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 940e082</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Local Supabase stack (supabase start) runs for INT-01 (ENV-02 card).</t>
+          <t>TC-06: analyst A requests node B's alerts through the Data API: no rows returned; no private data in errors.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>At 10:53 the Docker engine was not running (npx supabase status: exit 1, 'failed to inspect container health'). After Docker Desktop started: npx supabase start exit 0 (13:02:37), npx supabase status exit 0; db, auth, rest, storage, realtime, kong, studio, pg_meta, inbucket and analytics up. But supabase start listed the Edge Runtime under 'Stopped services' although supabase/config.toml enables it: its container had exited (255) 11 days earlier and was not restarted. The stack was therefore not complete. (This row was first logged as Pass at 13:03; corrected at 13:31 after INT-01.1 showed the cause.)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>DEF-02</t>
-        </is>
-      </c>
+          <t>Pilot hosted RLS check, read-only, each account under the authenticated role with its own JWT subject, 2026-10-16: 'cel.hendrix (Administrator) - both nodes: 467 on PC A and 1,527 on PC B'; 'celpca (PC A analyst) - PC A only (467); PC B's node row is not visible'; 'bryntpcb (PC B analyst) - PC B only'. UI: the Administrator's Alert History on PC A showed only PC A's alerts (ordinary pages default to the installation's own node; finding 6).</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/supabase-status.log; test-results/env_20261019/supabase-start.log; test-results/env_20261019/edge-runtime-restart.log; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §3 'Administrator reads across nodes'; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:04</t>
+          <t>2026-10-16 17:32 (pilot)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.1</t>
+          <t>SYS-03.P4</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>SYS-03</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Cel Hendrix N. San Miguel</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 9e18f30 (PC B) = 940e082 + test-cycle files</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Windows 11 test PC as in plan 5.1 (PC A: Intel Core i5-13420H, 16 GB RAM, Intel Wi-Fi 6 AX203).</t>
+          <t>Disconnect and reconnect: pending events kept and synced once (SYS-03 card).</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Home Single Language, version 26H2, OS build 26300.9711; host SANMIGUEL; Intel Core i5-13420H; 15.7 GB usable RAM; Intel Wi-Fi 6 AX203 (Up). The legacy registry field ProductName still reads 'Windows 10 Home Single Language'; the OS caption reads Windows 11.</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
+          <t>Pilot Test E, 2026-10-16, PC B: capture 12 started online at 09:29:04Z, went offline ~2 s later; 'It classified 210 flows offline, all held as pending.' 'Restarting offline refused sign-in, as designed.' bryntpcb signed in at 09:32:39Z; 'All 210 records were acknowledged between 09:32:44.6Z and 09:32:48.7Z, the last 9.5 s after sign-in. The cloud holds 210 events with 210 distinct event UUIDs, 210 traffic rows, 210 predictions and 139 alerts, all under PC B's node and owner. No PC A record changed.'</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1030,47 +1030,47 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §3 'Test E'; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:04</t>
+          <t>2026-10-16 17:32 (pilot)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.2</t>
+          <t>PRF-01.P8</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 9e18f30 (PC B)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>venv runs Python 3.14.6 with the library versions in requirements-model.lock (plan 5.1).</t>
+          <t>Pilot budget: outage recovery - all pending synced &lt;= 2 min after reconnect; 0 lost; 0 duplicates.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>venv\Scripts\python.exe = Python 3.14.6. numpy 2.5.1, scipy 1.18.0, pandas 3.0.3, scikit-learn 1.9.0, joblib 1.5.3, threadpoolctl 3.6.0 installed, each equal to requirements-model.lock.</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
+          <t>PC B: '9.5 s after sign-in; 0 lost; 0 duplicates'. Pilot verdict: 'Met. Timed from sign-in, because uploads after a restart wait for an online sign-in by design'.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1078,47 +1078,47 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/environment.txt; test-results/env_20261019/pip-freeze.txt; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:04</t>
+          <t>2026-10-16 17:40 (pilot)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.5</t>
+          <t>SYS-03.P3</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>SYS-03</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Cel Hendrix N. San Miguel</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 9e18f30 (PC B) = 940e082 + test-cycle files</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Npcap installed (plan 5.1).</t>
+          <t>TC-07: administrator revokes analyst B; B's prediction and capture refused; Restore re-enables.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Npcap 1.88 installed; npcap service Running (start type System); C:\Windows\System32\Npcap present.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+          <t>Pilot Test F, 2026-10-16: 'The Administrator revoked bryntpcb on PC B's node at 09:40:58Z and restored it at 09:45:21Z, then revoked and restored once more at 09:50:38Z and 09:50:42Z. While revoked, PC B was refused, and the cloud accepted no capture and no event from it. The exact wording on PC B was not recorded. After Restore, PC B still refused to monitor until Retry uploads was pressed on its Dashboard.' Five Starts during the block opened empty captures 13-17 (finding 5, Low, routed to 6C.1). 'After Retry uploads, capture 18 ran normally: 332 flows, 234 stored.' Prediction while revoked is not separately recorded.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1126,47 +1126,47 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §3 'Test F' and §5 finding 5; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:04</t>
+          <t>2026-10-16 17:40 (pilot)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.6</t>
+          <t>PRF-01.P9</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>dafe5e5</t>
+          <t>pilot 9e18f30 (PC B)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Administrator rights available for live capture (plan 5.1).</t>
+          <t>Pilot budget: revocation / restore - refused on the next action; works again after restore.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>The Windows account is a member of BUILTIN\Administrators. The terminal used for the automated runs is not elevated (Medium integrity), so it runs with RUN_WINDOWS_CAPTURE_TESTS unset; live capture needs scripts\START_APP.cmd started with 'Run as administrator'.</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
+          <t>PC B: 'refused immediately; works after Retry uploads'. Pilot verdict: 'Met, with the Retry uploads step now in the runbook'.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1174,29 +1174,29 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
+          <t>docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:26</t>
+          <t>2026-10-19 10:45</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>TC-13</t>
+          <t>ENV-01.3</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>UNT-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Cel Hendrix N. San Miguel</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1206,15 +1206,15 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>All tests pass; 0 lint and type errors (pytest -q; ruff check .; npm run typecheck; node --test tests/monitor_poll.test.cjs).</t>
+          <t>pip install -r requirements-dev.txt succeeds.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>pytest -q: 537 passed, 67 deselected (integration lane) in 130.13 s. ruff: All checks passed. pyright: 0 errors, 0 warnings, 0 informations. node --test monitor_poll: 11 pass, 0 fail. No flaky failures, so no re-run was needed. Run with RUN_WINDOWS_CAPTURE_TESTS=0 (terminal not elevated). The runner's 'uncommitted changes' flag refers only to the untracked docs/testing/ and test-results/ records.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
+          <t>Exit code 0. Every requirement was already satisfied; nothing changed.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1222,29 +1222,29 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>test-results/suites_20261019_132412/summary.md and pytest-offline.log, ruff-lint.log, pyright-typecheck.log, node-monitor-poll.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/pip-install-requirements-dev.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:27</t>
+          <t>2026-10-19 10:45</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>INT-01.1</t>
+          <t>ENV-01.4</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>INT-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1254,44 +1254,40 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Integration lane (pytest -m integration) passes against the local Supabase stack (INT-01 card).</t>
+          <t>pip install pytest-cov pip-audit bandit succeeds.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>5 failed, 60 passed, 2 skipped, 537 deselected in 54.27 s. All 5 failures are Edge Function calls answered HTTP 503 'name resolution failed' (test_enrollment_administration x4, test_local_supabase_stack::test_edge_function_smoke), because the local Edge Runtime container was not running (DEF-02). Test-environment fault; no product code involved.</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>DEF-02</t>
-        </is>
-      </c>
+          <t>Exit code 0. Installed pytest-cov 7.1.0 and coverage 7.16.2; pip-audit 2.10.1 and bandit 1.9.4 were already installed.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>test-results/suites_20261019_132412/pytest-integration.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/pip-install-test-tools.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:28</t>
+          <t>2026-10-19 10:45</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SEC-01.1</t>
+          <t>ENV-01.7</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1306,15 +1302,15 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>pip-audit finds no known vulnerability in requirements.txt, or each finding is fixed or justified (SEC-01 card).</t>
+          <t>Bundled datasets present and row counts recorded; UNSW_NB15_training-set.csv has 82,332 rows.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>python -m pip_audit -r requirements.txt: 'No known vulnerabilities found'.</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
+          <t>datasets/algoguard_big.csv 5,000 rows (1,597 Normal / 3,403 Attack); algoguard_bigger.csv 10,000 (3,194 / 6,806); algoguard_biggest.csv 20,000 (6,388 / 13,612); research/dataset/raw/UNSW_NB15_training-set.csv 82,332 rows, 45 columns (37,000 Normal / 45,332 Attack). SHA-256 of each file recorded.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1322,29 +1318,29 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>test-results/suites_20261019_132412/pip-audit.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/dataset_counts.json; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:29</t>
+          <t>2026-10-19 10:46</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ENV-02.2</t>
+          <t>ENV-01.8</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ENV-02</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1354,44 +1350,40 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Local Supabase stack (supabase start) runs for INT-01 (ENV-02 card).</t>
+          <t>Independent evaluation set built from the UNSW-NB15 training set with every row seen in training removed; row counts recorded (plan 5.1).</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Re-check after docker start supabase_edge_runtime_AlgoGuard (13:29:25): container Up; serving account_admin and smoke_test on 127.0.0.1:54321/functions/v1. All configured services running.</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
+          <t>82,332 rows loaded; 29,089 removed because their 15 features match a row in datasets/*.csv; 53,243 kept (20,674 Attack / 32,569 Normal). Generic attacks fall from 18,871 to 802 rows after removal; 7,387 kept rows repeat the features of another kept row.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>DEF-02</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/edge-runtime-restart.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/independent_set_counts.json (built with scripts/evaluate_model.py row_keys()); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:30</t>
+          <t>2026-10-19 10:51</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>INT-01.1</t>
+          <t>TC-16</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>INT-01</t>
+          <t>ENV-02</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1406,49 +1398,45 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Integration lane (pytest -m integration) passes against the local Supabase stack (INT-01 card).</t>
+          <t>Line coverage of services/ &gt;= 80% (pytest --cov=services).</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Re-run after the Edge Runtime restart: 65 passed, 2 skipped, 537 deselected in 43.70 s; exit 0. The 2 skips are the Npcap capture tests (INT-01.2).</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
+          <t>TOTAL 1,869 statements, 312 missed: 83% line coverage. 537 passed, 67 deselected (integration lane), 18 warnings (all ResourceWarning: unclosed sqlite3 connection, from test_live_monitor and test_model_architecture) in 290.45 s. Below 80% per module: traffic_source_service 69%, deployment_service 77%.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>DEF-02</t>
-        </is>
-      </c>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
+          <t>test-results/coverage_20261019_104655/pytest-cov.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:30</t>
+          <t>2026-10-19 13:00</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>INT-01.2</t>
+          <t>ENV-01.9</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>INT-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1458,15 +1446,15 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Npcap capture integration tests (test_cloud_app_stack live capture, test_maintenance_capture) pass with RUN_WINDOWS_CAPTURE_TESTS=1.</t>
+          <t>Official UNSW_NB15_testing-set.csv (175,341 rows) in research/dataset/raw/ for model B (SYS-01).</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Not executed: both skipped ('Set RUN_WINDOWS_CAPTURE_TESTS=1 on Windows with Npcap.') because the automated runs use a terminal that is not elevated. Can be run from an elevated Command Prompt.</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+          <t>Not executed: the file is not on this PC (checked 10:45 and 13:00). An alternative for the model B comparison is to be decided at Checkpoint 1.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Not executed</t>
         </is>
@@ -1474,29 +1462,29 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/dataset_counts.json; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 13:50</t>
+          <t>2026-10-19 13:00</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ENV-02.1</t>
+          <t>ENV-01.10</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>ENV-02</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1506,49 +1494,45 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
+          <t>Second PC for the two-PC pilot confirmed, or reported unavailable to the Test Lead (ENV-01 card).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Re-check with the job logs (gh signed in). Both runs (cb3bcdb 38886300881, 940e082 38870178965): setup-python 'python-version: 3.14' installed CPython 3.14.8; Lint 'All checks passed!'; Type check '0 errors, 26 warnings' (all 26 reportMissingModuleSource for maintainer-only packages); Unit tests '5 failed, 476 passed, 21 skipped, 34 deselected, 40 errors'. 44 of the 45 failures/errors are model_runtime.ModelDeliveryError ('Install the locked Python model runtime' x43, 'Retrain this artifact with the locked model runtime' x1): verify_runtime() requires exactly Python 3.14.6 (DEF-01). The 45th is test_cloud_outbox.py::test_cap_reserves_before_enqueue_and_retry_does_not_consume_slot, 'assert spool.drain()' False at line 55 in both runs (DEF-03).</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>DEF-01, DEF-03</t>
-        </is>
-      </c>
+          <t>PC B is not available on 2026-10-19. Reported in this log and in the Test Status Report (DOC-05). Plan section 8 contingency applies: SYS-03 hardware steps Not executed; the automated two-node integration tests (INT-01) cover isolation.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>test-results/env_20261019/ci_run_38886300881_cb3bcdb_failed.log; test-results/env_20261019/ci_run_38870178965_940e082_failed.log (gh run view --log-failed)</t>
+          <t>Lead Architect's answer, 2026-10-19 13:00; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:05</t>
+          <t>2026-10-19 13:00</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ENV-01.11</t>
+          <t>ENV-02.1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>ENV-02</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1558,45 +1542,49 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>App starts on 127.0.0.1:5000 in cloud mode (ENV-01 card; local mode is checked separately in SEC-01 / TC-10).</t>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>scripts\START_APP.cmd started python app.py at 15:02:30 (2 processes: venv launcher + interpreter). GET http://127.0.0.1:5000/login -&gt; HTTP 200 'Login | AlgoGuard', heading 'Cloud Pilot Access', e-mail + password form (cloud sign-in). Model cache C:\AlgoGuardPilot\state-PC-A\models holds only 1-9c9f0fb1...joblib (SHA-256 9c9f0fb18524eeda...).</t>
+          <t>CI workflow (windows-latest) failed on cb3bcdb (run 38886300881, 2026-10-16) and on 940e082 (runs 38870178965 on 2026-10-16 and 38017196080 on 2026-10-10). In both 2026-10-16 runs: Lint success, Type check success, Unit tests failure ('Process completed with exit code 1'), Browser polling tests skipped. All six runs listed for main (back to 4c9666c, 2026-10-05) concluded failure.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>DEF-01</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Session check of the /login page and the model cache folder (no credentials read); evidence: product code = 940e082</t>
+          <t>GitHub REST API (unauthenticated) actions/runs and jobs for main; job logs need sign-in (HTTP 403); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:23</t>
+          <t>2026-10-19 13:03</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>TC-01</t>
+          <t>ENV-02.2</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>SMK-01</t>
+          <t>ENV-02</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>John Brian A. Tiopes</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1606,45 +1594,49 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Known Normal row from algoguard_big.csv on Manual Prediction: verdict Normal; event saved.</t>
+          <t>Local Supabase stack (supabase start) runs for INT-01 (ENV-02 card).</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Input: first Normal row of datasets/algoguard_big.csv (CSV line 2). Signed in as the PC A analyst, cloud mode. Result: NORMAL, model confidence 84.11%; Model Stacking Ensemble; Deployment #1; latency 147.987 ms; event b0087c8e-f95c-4ce9-aa80-bfa0422f8f73; page: 'Saved on this computer - pending upload', Prediction 'Assigned after upload', Alert 'Not created'. Outbox (read-only, 15:23): event created 15:22:59, status synced, receipt prediction_id 2913, alert_id null, node d535e2fd (PC A), deployment 1.</t>
+          <t>At 10:53 the Docker engine was not running (npx supabase status: exit 1, 'failed to inspect container health'). After Docker Desktop started: npx supabase start exit 0 (13:02:37), npx supabase status exit 0; db, auth, rest, storage, realtime, kong, studio, pg_meta, inbucket and analytics up. But supabase start listed the Edge Runtime under 'Stopped services' although supabase/config.toml enables it: its container had exited (255) 11 days earlier and was not restarted. The stack was therefore not complete. (This row was first logged as Pass at 13:03; corrected at 13:31 after INT-01.1 showed the cause.)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>DEF-02</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>test-results/smoke_20261019/TC-01_manual_normal.png; local outbox C:\AlgoGuardPilot\state-PC-A\outbox\outbox.sqlite3 (read-only query); evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/supabase-status.log; test-results/env_20261019/supabase-start.log; test-results/env_20261019/edge-runtime-restart.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:29</t>
+          <t>2026-10-19 13:04</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>TC-02</t>
+          <t>ENV-01.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>SMK-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>John Brian A. Tiopes</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1654,15 +1646,15 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Known Attack row from algoguard_big.csv on Manual Prediction: verdict Attack; alert created with confidence.</t>
+          <t>Windows 11 test PC as in plan 5.1 (PC A: Intel Core i5-13420H, 16 GB RAM, Intel Wi-Fi 6 AX203).</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Input: first Attack row of datasets/algoguard_big.csv (CSV line 3). Result: ATTACK, model confidence 92.95%; Model Stacking Ensemble; Deployment #1; latency 44.745 ms; event 5a86608a-76da-41c6-ba68-4c63e7eccbcb; page: 'Saved on this computer - pending upload', Alert 'Created when the record uploads'. Outbox (read-only, 15:29): event created 15:29:25, status synced, receipt prediction_id 2914, alert_id 2319, node d535e2fd (PC A), deployment 1.</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
+          <t>Microsoft Windows 11 Home Single Language, version 26H2, OS build 26300.9711; host SANMIGUEL; Intel Core i5-13420H; 15.7 GB usable RAM; Intel Wi-Fi 6 AX203 (Up). The legacy registry field ProductName still reads 'Windows 10 Home Single Language'; the OS caption reads Windows 11.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1670,29 +1662,29 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>test-results/smoke_20261019/TC-02_manual_attack.png; local outbox (read-only query); evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:35</t>
+          <t>2026-10-19 13:04</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>SMK-01.3</t>
+          <t>ENV-01.2</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>SMK-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>John Brian A. Tiopes</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1702,15 +1694,15 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Short CSV replay produces alerts with no errors (SMK-01 card).</t>
+          <t>venv runs Python 3.14.6 with the library versions in requirements-model.lock (plan 5.1).</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Live Monitor, Sample replay algoguard_big.csv (5,000 flows), Fast, Sequential, Save attacks; stopped after 386 of 5,000 flows. Screen: Flows Analyzed 386; Attacks 275 (71.24%); Normal 111; Alerts Queued 275; average latency 130.725 ms; Pinned deployment #1; Label mismatches 15; Queued for upload 275; Synced to cloud 275; Pending upload 0; Not stored 0; Upload status active; no error message. Outbox (read-only, 15:35): session c89500d0 holds 275 events, all synced, all 275 receipts carry an alert_id, 15:31:20-15:34:30, deployment 1, node d535e2fd. Observation for USE-01: the Recent Flows time column shows UTC (07:34:30 for 15:34:30 local) without a label.</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
+          <t>venv\Scripts\python.exe = Python 3.14.6. numpy 2.5.1, scipy 1.18.0, pandas 3.0.3, scikit-learn 1.9.0, joblib 1.5.3, threadpoolctl 3.6.0 installed, each equal to requirements-model.lock.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1718,29 +1710,29 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>test-results/smoke_20261019/SMK-01_csv_replay_counters.png and SMK-01_csv_replay_sidepanel.png; local outbox (read-only query); evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/environment.txt; test-results/env_20261019/pip-freeze.txt; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:37</t>
+          <t>2026-10-19 13:04</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>TC-03</t>
+          <t>ENV-01.5</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1750,49 +1742,45 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Whole independent set through the saved pipeline: accuracy, F1, attack recall &gt;= 90%; FPR &lt;= 8%; ROC-AUC &gt;= 0.95 (plan 3.3).</t>
+          <t>Npcap installed (plan 5.1).</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Model A = deployed Stacking Ensemble (saved_models/run_3/stacking.joblib, SHA-256 9c9f0fb1...847c = deployment #1, trained 2026-10-08 on algoguard_big.csv). Independent set: 82,332 loaded, 29,089 removed as seen, 53,243 evaluated (20,674 attack / 32,569 normal). Accuracy 81.47% (not met), F1 79.49% (not met), recall 92.44% (met), FPR 25.49% (not met), ROC-AUC 0.9371 (not met); precision 69.72%, specificity 74.51%. Confusion: TN 24,268, FP 8,301, FN 1,563, TP 19,111. Harness check: the same model and code on algoguard_big.csv (seen data) give accuracy 96.98%, F1 97.77%, FPR 4.07%, ROC-AUC 0.9963, so the drop is a generalisation gap, not a scoring error.</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>DEF-04, DEF-05, DEF-06, DEF-07</t>
-        </is>
-      </c>
+          <t>Npcap 1.88 installed; npcap service Running (start type System); C:\Windows\System32\Npcap present.</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>test-results/evaluation_20261019_153649/ (summary.md, metrics.json, confusion_matrix.csv, console.log, sanity_seen_rows.log); evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:37</t>
+          <t>2026-10-19 13:04</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>SYS-01.2</t>
+          <t>ENV-01.6</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1802,15 +1790,15 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Stacking compared with each single model on the same rows (F1, ROC-AUC, time per row) (SYS-01 card).</t>
+          <t>Administrator rights available for live capture (plan 5.1).</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Same 53,243 rows. F1 / ROC-AUC / ms per row: Random Forest 0.7957 / 0.9306 / 0.0096; Stacking 0.7949 / 0.9371 / 0.0836; Gradient Boosting 0.7765 / 0.9292 / 0.0037; KNN 0.7629 / 0.8962 / 0.0086; AdaBoost 0.7444 / 0.8907 / 0.0315; Naive Bayes 0.3130 / 0.6108 / 0.0036. Stacking has the best ROC-AUC and ties Random Forest on accuracy (0.8147); Random Forest is marginally higher on F1 and recall. Comparison recorded.</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
+          <t>The Windows account is a member of BUILTIN\Administrators. The terminal used for the automated runs is not elevated (Medium integrity), so it runs with RUN_WINDOWS_CAPTURE_TESTS unset; live capture needs scripts\START_APP.cmd started with 'Run as administrator'.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1818,29 +1806,29 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>test-results/evaluation_20261019_153649/model_comparison.csv; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/environment.txt; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:37</t>
+          <t>2026-10-19 13:26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>SYS-01.3</t>
+          <t>TC-13</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>UNT-01</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Cel Hendrix N. San Miguel</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1850,15 +1838,15 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Recall per attack category measured; categories below 90% flagged (SYS-01 card).</t>
+          <t>All tests pass; 0 lint and type errors (pytest -q; ruff check .; npm run typecheck; node --test tests/monitor_poll.test.cjs).</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Recall: Analysis 99.76%, Reconnaissance 99.71%, Exploits 98.00%, Backdoor 97.78%, DoS 96.93%, Worms 95.35% (43 rows), Generic 91.27% (802 rows). FLAGGED below 90%: Fuzzers 76.62% (5,064 rows) and Shellcode 89.97% (359 rows). Normal specificity 74.51% (32,569 rows).</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
+          <t>pytest -q: 537 passed, 67 deselected (integration lane) in 130.13 s. ruff: All checks passed. pyright: 0 errors, 0 warnings, 0 informations. node --test monitor_poll: 11 pass, 0 fail. No flaky failures, so no re-run was needed. Run with RUN_WINDOWS_CAPTURE_TESTS=0 (terminal not elevated). The runner's 'uncommitted changes' flag refers only to the untracked docs/testing/ and test-results/ records.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1866,29 +1854,29 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>test-results/evaluation_20261019_153649/per_category.csv; evidence: product code = 940e082</t>
+          <t>test-results/suites_20261019_132412/summary.md and pytest-offline.log, ruff-lint.log, pyright-typecheck.log, node-monitor-poll.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:39</t>
+          <t>2026-10-19 13:27</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>SYS-01.4</t>
+          <t>INT-01.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>INT-01</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1898,45 +1886,49 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Re-run with the same seed gives the same numbers (SYS-01 card).</t>
+          <t>Integration lane (pytest -m integration) passes against the local Supabase stack (INT-01 card).</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Model A retrained the same way: python train.py datasets/algoguard_big.csv --models-dir saved_models/cycle1_A2 (local run 4, 16.1 s, no --deploy; Stacking test-split F1 95.07%, as recorded for model A). Artifact 8,558,646 bytes, SHA-256 5fc6ee7c... (differs from A only by its stored run metadata). On the independent set: accuracy 0.8147, F1 0.7949, recall 0.9244, FPR 0.2549, ROC-AUC 0.9371, confusion 24,268 / 8,301 / 1,563 / 19,111 - identical to A. Row by row on 53,243 rows: 0 verdicts differ; max attack-probability difference 0.0.</t>
+          <t>5 failed, 60 passed, 2 skipped, 537 deselected in 54.27 s. All 5 failures are Edge Function calls answered HTTP 503 'name resolution failed' (test_enrollment_administration x4, test_local_supabase_stack::test_edge_function_smoke), because the local Edge Runtime container was not running (DEF-02). Test-environment fault; no product code involved.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>DEF-02</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>test-results/evaluation_20261019_153850/ (summary.md, console.log, train_A2_console.log, A_vs_A2_row_by_row.json); evidence: product code = 940e082</t>
+          <t>test-results/suites_20261019_132412/pytest-integration.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:50</t>
+          <t>2026-10-19 13:28</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SYS-01.5</t>
+          <t>SEC-01.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1946,49 +1938,45 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Model B (comparison only) trained from the UNSW-NB15 training file with train.py, no --deploy, training time recorded; usable for an A-vs-B comparison on unseen data (Master Prompt Phase 4).</t>
+          <t>pip-audit finds no known vulnerability in requirements.txt, or each finding is fixed or justified (SEC-01 card).</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Official testing set unavailable, so B was trained on the training file minus a seeded 30% key-group hold-out (66,393 rows; hold-out 15,939 rows, 0 overlap). python train.py research/dataset/processed/sys01_holdout/model_b_train.csv --models-dir saved_models/cycle1_B: local run 5, 152 s, exit 0. train.py used all 44 non-target columns as features, including attack_cat (encodes the label) and id; Random Forest, AdaBoost, Gradient Boosting, Naive Bayes and Stacking all reported 100.00% accuracy / F1 / ROC-AUC (Naive Bayes scored 48.72% on model A's data). evaluate_model.py refused the artifact ('expects different features'). Not usable; a 15-feature model B was trained instead (SYS-01.6).</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>DEF-08</t>
-        </is>
-      </c>
+          <t>python -m pip_audit -r requirements.txt: 'No known vulnerabilities found'.</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>test-results/sys01_holdout/train_B_console.log, eval_B_raw_console.log, holdout_manifest.json; saved_models/cycle1_B/run_5 (git-ignored); evidence: product code = 940e082</t>
+          <t>test-results/suites_20261019_132412/pip-audit.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 15:59</t>
+          <t>2026-10-19 13:29</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>SYS-01.6</t>
+          <t>ENV-02.2</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>SYS-01</t>
+          <t>ENV-02</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Victor Alexander A. Ong</t>
+          <t>Afel Anthonielle V. Quirao</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1998,35 +1986,39 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Comparison only (not the official result): model A and model B evaluated on the same unseen rows (Master Prompt Phase 4, adapted: hold-out instead of the official testing set).</t>
+          <t>Local Supabase stack (supabase start) runs for INT-01 (ENV-02 card).</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Model B = 15-feature retrain on the same 66,393 rows (local run 6, 809.9 s; test-split Stacking F1 95.42%). Hold-out 15,939 rows (6,174 attack / 9,765 normal), 0 removed as seen by either model. A: accuracy 81.69%, F1 79.56%, recall 92.03%, FPR 24.85%, ROC-AUC 0.9375, 0.144 ms/row. B: accuracy 90.79%, F1 87.36%, recall 82.18%, FPR 3.77%, ROC-AUC 0.9713, 0.236 ms/row. B cuts false positives (2,427 -&gt; 368) but misses more attacks (492 -&gt; 1,100 FN); B recall Fuzzers 49.47%, Shellcode 59.29%. A on the hold-out matches its official 53,243-row result within 0.6 points.</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
+          <t>Re-check after docker start supabase_edge_runtime_AlgoGuard (13:29:25): container Up; serving account_admin and smoke_test on 127.0.0.1:54321/functions/v1. All configured services running.</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>DEF-02</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>test-results/sys01_holdout/ (eval_A_on_holdout/, eval_B_on_holdout/, *_console.log, holdout_manifest.json, model_b_train_15_manifest.json, train_B15_console.log, make_holdout.py, make_b15.py); evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/edge-runtime-restart.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 16:16</t>
+          <t>2026-10-19 13:30</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>INT-01.3</t>
+          <t>INT-01.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2046,35 +2038,39 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Preprocessing to Stacking to alert path verified; Stacking uses all five base models and the Logistic Regression final estimator; model delivery, publication and outbox unit tests pass (INT-01 card).</t>
+          <t>Integration lane (pytest -m integration) passes against the local Supabase stack (INT-01 card).</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>pytest -q tests/test_model_delivery.py tests/test_model_publication.py tests/test_cloud_outbox.py tests/test_model_architecture.py: 42 passed in 39.49 s (includes test_stacking_uses_five_models_and_logistic_regression). Deployed artifact (run_3/stacking.joblib, SHA-256 9c9f0fb1...): pipeline preprocessor -&gt; StackingClassifier with fitted RandomForestClassifier, GradientBoostingClassifier, AdaBoostClassifier, KNeighborsClassifier, GaussianNB; final estimator LogisticRegression; cv 5, predict_proba stacking. End-to-end path to alert shown by TC-02 (alert #2319).</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
+          <t>Re-run after the Edge Runtime restart: 65 passed, 2 skipped, 537 deselected in 43.70 s; exit 0. The 2 skips are the Npcap capture tests (INT-01.2).</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>DEF-02</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>test-results/int01_20261019_161543/pytest-int01-units.log, inspect_stacking_modelA.log, inspect_stacking.py; evidence: product code = 940e082</t>
+          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:03</t>
+          <t>2026-10-19 13:30</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>TC-08</t>
+          <t>INT-01.2</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2094,44 +2090,40 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>One byte changed in the cached artifact (local copy, backed up); app restarted: SHA-256 mismatch reported; model not loaded.</t>
+          <t>Npcap capture integration tests (test_cloud_app_stack live capture, test_maintenance_capture) pass with RUN_WINDOWS_CAPTURE_TESTS=1.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>App stopped 16:58 (outbox 919 synced, 0 pending). Cache backed up to C:\AlgoGuardPilot\TC08-backup-models-20261019 (SHA-256 verified equal). Byte at offset 4,279,323 of 1-9c9f0fb1...joblib changed 0x00 -&gt; 0x01 (SHA-256 now c8f1c7fe..., size unchanged). App restarted 17:00:30, PC A analyst signed in. Predict page: 'No active deployment - The cached model is corrupt. Remove it and retry.'; no form, no prediction possible. Live Monitor: the same message, no capture controls. The app neither deleted nor replaced the file. Dashboard still showed the cloud deployment as 'Deployed' with no local warning (DEF-09, Low).</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>DEF-09</t>
-        </is>
-      </c>
+          <t>Not executed: both skipped ('Set RUN_WINDOWS_CAPTURE_TESTS=1 on Windows with Npcap.') because the automated runs use a terminal that is not elevated. Can be run from an elevated Command Prompt.</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>test-results/int01_20261019_161543/tc08_corruption.json, TC-08_predict_refused.png, TC-08_live_monitor_refused.png, TC-08_dashboard_while_corrupt.png, tc08_flip_byte.py; evidence: product code = 940e082</t>
+          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:12</t>
+          <t>2026-10-19 13:50</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>TC-08</t>
+          <t>ENV-02.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>INT-01</t>
+          <t>ENV-02</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2146,45 +2138,49 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>After restoring the backup, the app loads the model again (Master Prompt Phase 5.3).</t>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>App stopped; backup copied back at 17:07; cached file SHA-256 9c9f0fb1...847c again (8,558,646 bytes, only file in the cache). App restarted as administrator, PC A analyst signed in. Predict form shown again; Run Prediction: green verdict at 50.46% confidence, Stacking Ensemble, Deployment #1, latency 2,021.727 ms (first prediction after start), event 3f69afc9..., synced as prediction #3190, no alert. The confidence differs from TC-01 (84.11%): the screenshot shows sinpkt typed as 133.42319, but offline re-scoring of the exact row and of that variant both give Normal 84.11%, so another typed value (not visible, and cleared from the outbox after sync) probably differed. Not counted as a defect; the model loaded and classified.</t>
+          <t>Re-check with the job logs (gh signed in). Both runs (cb3bcdb 38886300881, 940e082 38870178965): setup-python 'python-version: 3.14' installed CPython 3.14.8; Lint 'All checks passed!'; Type check '0 errors, 26 warnings' (all 26 reportMissingModuleSource for maintainer-only packages); Unit tests '5 failed, 476 passed, 21 skipped, 34 deselected, 40 errors'. 44 of the 45 failures/errors are model_runtime.ModelDeliveryError ('Install the locked Python model runtime' x43, 'Retrain this artifact with the locked model runtime' x1): verify_runtime() requires exactly Python 3.14.6 (DEF-01). The 45th is test_cloud_outbox.py::test_cap_reserves_before_enqueue_and_retry_does_not_consume_slot, 'assert spool.drain()' False at line 55 in both runs (DEF-03).</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>DEF-01, DEF-03</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>test-results/int01_20261019_161543/TC-08_after_restore_prediction.png, tc08_recheck_row.py, tc08_recheck_row.log; evidence: product code = 940e082</t>
+          <t>test-results/env_20261019/ci_run_38886300881_cb3bcdb_failed.log; test-results/env_20261019/ci_run_38870178965_940e082_failed.log (gh run view --log-failed)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:21</t>
+          <t>2026-10-19 15:05</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>ENV-01.11</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>INT-01</t>
+          <t>ENV-01</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Afel Anthonielle V. Quirao</t>
+          <t>Arella Biacea B. Mirasol</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2194,15 +2190,15 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>CSV replay running in cloud mode; disconnect, restart, reconnect, sign in: pending events kept and synced once; no duplicates.</t>
+          <t>App starts on 127.0.0.1:5000 in cloud mode (ENV-01 card; local mode is checked separately in SEC-01 / TC-10).</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Baseline 17:15: outbox 920 synced, 0 pending. Live Monitor replay (algoguard_big, Fast, Sequential, Save every flow) started; Wi-Fi switched off (not Airplane mode). Offline: new flows marked Pending; side panel Queued 142, Synced 39, Pending 103, Not stored 0, Upload status 'retrying (transient)'. Capture stopped and app closed offline; app restarted offline: sign-in refused with 'The cloud is unreachable. Online sign-in is required; a cached model does not permit offline access.' (by design); a page showed 'The cloud is unavailable. Pending records stay on this computer.' Wi-Fi on, signed in: Dashboard 17:21 showed Pending 63 durable, Synced 417, Rejected 0, Not stored 0. Outbox 17:21:28: capture session 4ea6f1f9 holds 202 events (17:17:43-17:19:28), all synced, 0 pending; outbox total 1,122 = 920 + 202. 202 distinct event UUIDs and 202 distinct cloud prediction ids, contiguous #3191-#3392; 145 distinct alert ids. No duplicates, none lost.</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
+          <t>scripts\START_APP.cmd started python app.py at 15:02:30 (2 processes: venv launcher + interpreter). GET http://127.0.0.1:5000/login -&gt; HTTP 200 'Login | AlgoGuard', heading 'Cloud Pilot Access', e-mail + password form (cloud sign-in). Model cache C:\AlgoGuardPilot\state-PC-A\models holds only 1-9c9f0fb1...joblib (SHA-256 9c9f0fb18524eeda...).</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2210,29 +2206,29 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>test-results/int01_20261019_161543/TC-09_*.png (sign-in screenshot e-mail redacted), tc09_outbox_check.json, tc09_outbox_sessions.txt; evidence: product code = 940e082</t>
+          <t>Session check of the /login page and the model cache folder (no credentials read); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:24</t>
+          <t>2026-10-19 15:23</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>SEC-01.2</t>
+          <t>TC-01</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SMK-01</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>John Brian A. Tiopes</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2242,15 +2238,15 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>CSRF: missing or forged tokens refused; sign-in throttle logic (SEC-01 card; Master Prompt: pytest tests/test_api_validation.py tests/test_login_throttle.py).</t>
+          <t>Known Normal row from algoguard_big.csv on Manual Prediction: verdict Normal; event saved.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>25 passed in 31.52 s: invalid JSON bodies rejected before any action (16 cases), JSON actions require a JSON content type (2), invalid or forged login tokens return a client error (3); throttle: repeated failures pause the account then release it, success clears the counter, one address cannot spray many usernames, old failures are forgotten. Cookie writes without a CSRF token are also covered by tests/test_cloud_app.py::test_cookie_writes_require_csrf_but_bearer_api_calls_do_not, which passed in TC-13.</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
+          <t>Input: first Normal row of datasets/algoguard_big.csv (CSV line 2). Signed in as the PC A analyst, cloud mode. Result: NORMAL, model confidence 84.11%; Model Stacking Ensemble; Deployment #1; latency 147.987 ms; event b0087c8e-f95c-4ce9-aa80-bfa0422f8f73; page: 'Saved on this computer - pending upload', Prediction 'Assigned after upload', Alert 'Not created'. Outbox (read-only, 15:23): event created 15:22:59, status synced, receipt prediction_id 2913, alert_id null, node d535e2fd (PC A), deployment 1.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2258,29 +2254,29 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>test-results/sec01_20261019_172340/pytest-csrf-throttle.log; evidence: product code = 940e082</t>
+          <t>test-results/smoke_20261019/TC-01_manual_normal.png; local outbox C:\AlgoGuardPilot\state-PC-A\outbox\outbox.sqlite3 (read-only query); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:31</t>
+          <t>2026-10-19 15:29</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>SEC-01.3</t>
+          <t>TC-02</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SMK-01</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>John Brian A. Tiopes</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2290,15 +2286,15 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Bandit run; every Medium/High finding fixed or justified, or a defect raised (SEC-01 card; Master Prompt Phase 6).</t>
+          <t>Known Attack row from algoguard_big.csv on Manual Prediction: verdict Attack; alert created with confidence.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Bandit (13:28 scan) by severity: High 0, Medium 14, Low 18. All 14 Medium findings read in the source and justified as false positives: 3 x B104 are an outgoing socket bound to an ephemeral port before connect (cloud_connections.py:177, maintenance_connections.py:141) and a host-name list (maintainer_env.py:44) - nothing listens; 11 x B608 build SQL only from fixed table/column lists or '?' placeholders, with every value passed as a parameter (cloud_outbox.py, legacy_backup.py, legacy_import.py, database_service.py). Hardening suggestion (not a defect): call icacls by full path in cloud_outbox.py:55. No defect raised.</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
+          <t>Input: first Attack row of datasets/algoguard_big.csv (CSV line 3). Result: ATTACK, model confidence 92.95%; Model Stacking Ensemble; Deployment #1; latency 44.745 ms; event 5a86608a-76da-41c6-ba68-4c63e7eccbcb; page: 'Saved on this computer - pending upload', Alert 'Created when the record uploads'. Outbox (read-only, 15:29): event created 15:29:25, status synced, receipt prediction_id 2914, alert_id 2319, node d535e2fd (PC A), deployment 1.</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2306,29 +2302,29 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>test-results/sec01_20261019_172340/bandit_review.md; test-results/suites_20261019_132412/bandit.log; evidence: product code = 940e082</t>
+          <t>test-results/smoke_20261019/TC-02_manual_attack.png; local outbox (read-only query); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:33</t>
+          <t>2026-10-19 15:35</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>SEC-01.4</t>
+          <t>SMK-01.3</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>SMK-01</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Arella Biacea B. Mirasol</t>
+          <t>John Brian A. Tiopes</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2338,15 +2334,15 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Secrets: git ls-files lists only the .env .example files; git grep for sb_secret_ / service_role / JWT-like strings finds nothing outside tests/fixtures (Master Prompt Phase 6).</t>
+          <t>Short CSV replay produces alerts with no errors (SMK-01 card).</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Tracked .env files: .env.example and .env.maintainer.example only. git grep (HEAD): 21 hits, 0 JWT-like strings. Outside tests: service_role is the Postgres role name in 14 migration lines, supabase/config.toml:24 (comment) and docs/migration/05b-access.md:606 (prose); scripts/run_test_suites.py:37 is the redaction regex. Tests: test_cloud_schema.py, test_cloud_app.py, test_cloud_repository.py (fixtures). No secret values found; values were not printed.</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+          <t>Live Monitor, Sample replay algoguard_big.csv (5,000 flows), Fast, Sequential, Save attacks; stopped after 386 of 5,000 flows. Screen: Flows Analyzed 386; Attacks 275 (71.24%); Normal 111; Alerts Queued 275; average latency 130.725 ms; Pinned deployment #1; Label mismatches 15; Queued for upload 275; Synced to cloud 275; Pending upload 0; Not stored 0; Upload status active; no error message. Outbox (read-only, 15:35): session c89500d0 holds 275 events, all synced, all 275 receipts carry an alert_id, 15:31:20-15:34:30, deployment 1, node d535e2fd. Observation for USE-01: the Recent Flows time column shows UTC (07:34:30 for 15:34:30 local) without a label.</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2354,12 +2350,792 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
+          <t>test-results/smoke_20261019/SMK-01_csv_replay_counters.png and SMK-01_csv_replay_sidepanel.png; local outbox (read-only query); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:37</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Whole independent set through the saved pipeline: accuracy, F1, attack recall &gt;= 90%; FPR &lt;= 8%; ROC-AUC &gt;= 0.95 (plan 3.3).</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Model A = deployed Stacking Ensemble (saved_models/run_3/stacking.joblib, SHA-256 9c9f0fb1...847c = deployment #1, trained 2026-10-08 on algoguard_big.csv). Independent set: 82,332 loaded, 29,089 removed as seen, 53,243 evaluated (20,674 attack / 32,569 normal). Accuracy 81.47% (not met), F1 79.49% (not met), recall 92.44% (met), FPR 25.49% (not met), ROC-AUC 0.9371 (not met); precision 69.72%, specificity 74.51%. Confusion: TN 24,268, FP 8,301, FN 1,563, TP 19,111. Harness check: the same model and code on algoguard_big.csv (seen data) give accuracy 96.98%, F1 97.77%, FPR 4.07%, ROC-AUC 0.9963, so the drop is a generalisation gap, not a scoring error.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>DEF-04, DEF-05, DEF-06, DEF-07</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>test-results/evaluation_20261019_153649/ (summary.md, metrics.json, confusion_matrix.csv, console.log, sanity_seen_rows.log); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:37</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01.2</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Stacking compared with each single model on the same rows (F1, ROC-AUC, time per row) (SYS-01 card).</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Same 53,243 rows. F1 / ROC-AUC / ms per row: Random Forest 0.7957 / 0.9306 / 0.0096; Stacking 0.7949 / 0.9371 / 0.0836; Gradient Boosting 0.7765 / 0.9292 / 0.0037; KNN 0.7629 / 0.8962 / 0.0086; AdaBoost 0.7444 / 0.8907 / 0.0315; Naive Bayes 0.3130 / 0.6108 / 0.0036. Stacking has the best ROC-AUC and ties Random Forest on accuracy (0.8147); Random Forest is marginally higher on F1 and recall. Comparison recorded.</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>test-results/evaluation_20261019_153649/model_comparison.csv; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:37</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01.3</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Recall per attack category measured; categories below 90% flagged (SYS-01 card).</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Recall: Analysis 99.76%, Reconnaissance 99.71%, Exploits 98.00%, Backdoor 97.78%, DoS 96.93%, Worms 95.35% (43 rows), Generic 91.27% (802 rows). FLAGGED below 90%: Fuzzers 76.62% (5,064 rows) and Shellcode 89.97% (359 rows). Normal specificity 74.51% (32,569 rows).</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>test-results/evaluation_20261019_153649/per_category.csv; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:39</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01.4</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Re-run with the same seed gives the same numbers (SYS-01 card).</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Model A retrained the same way: python train.py datasets/algoguard_big.csv --models-dir saved_models/cycle1_A2 (local run 4, 16.1 s, no --deploy; Stacking test-split F1 95.07%, as recorded for model A). Artifact 8,558,646 bytes, SHA-256 5fc6ee7c... (differs from A only by its stored run metadata). On the independent set: accuracy 0.8147, F1 0.7949, recall 0.9244, FPR 0.2549, ROC-AUC 0.9371, confusion 24,268 / 8,301 / 1,563 / 19,111 - identical to A. Row by row on 53,243 rows: 0 verdicts differ; max attack-probability difference 0.0.</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>test-results/evaluation_20261019_153850/ (summary.md, console.log, train_A2_console.log, A_vs_A2_row_by_row.json); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:50</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01.5</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Model B (comparison only) trained from the UNSW-NB15 training file with train.py, no --deploy, training time recorded; usable for an A-vs-B comparison on unseen data (Master Prompt Phase 4).</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Official testing set unavailable, so B was trained on the training file minus a seeded 30% key-group hold-out (66,393 rows; hold-out 15,939 rows, 0 overlap). python train.py research/dataset/processed/sys01_holdout/model_b_train.csv --models-dir saved_models/cycle1_B: local run 5, 152 s, exit 0. train.py used all 44 non-target columns as features, including attack_cat (encodes the label) and id; Random Forest, AdaBoost, Gradient Boosting, Naive Bayes and Stacking all reported 100.00% accuracy / F1 / ROC-AUC (Naive Bayes scored 48.72% on model A's data). evaluate_model.py refused the artifact ('expects different features'). Not usable; a 15-feature model B was trained instead (SYS-01.6).</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>DEF-08</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sys01_holdout/train_B_console.log, eval_B_raw_console.log, holdout_manifest.json; saved_models/cycle1_B/run_5 (git-ignored); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:59</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01.6</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>SYS-01</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Victor Alexander A. Ong</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Comparison only (not the official result): model A and model B evaluated on the same unseen rows (Master Prompt Phase 4, adapted: hold-out instead of the official testing set).</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Model B = 15-feature retrain on the same 66,393 rows (local run 6, 809.9 s; test-split Stacking F1 95.42%). Hold-out 15,939 rows (6,174 attack / 9,765 normal), 0 removed as seen by either model. A: accuracy 81.69%, F1 79.56%, recall 92.03%, FPR 24.85%, ROC-AUC 0.9375, 0.144 ms/row. B: accuracy 90.79%, F1 87.36%, recall 82.18%, FPR 3.77%, ROC-AUC 0.9713, 0.236 ms/row. B cuts false positives (2,427 -&gt; 368) but misses more attacks (492 -&gt; 1,100 FN); B recall Fuzzers 49.47%, Shellcode 59.29%. A on the hold-out matches its official 53,243-row result within 0.6 points.</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sys01_holdout/ (eval_A_on_holdout/, eval_B_on_holdout/, *_console.log, holdout_manifest.json, model_b_train_15_manifest.json, train_B15_console.log, make_holdout.py, make_b15.py); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:16</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>INT-01.3</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>INT-01</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Preprocessing to Stacking to alert path verified; Stacking uses all five base models and the Logistic Regression final estimator; model delivery, publication and outbox unit tests pass (INT-01 card).</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>pytest -q tests/test_model_delivery.py tests/test_model_publication.py tests/test_cloud_outbox.py tests/test_model_architecture.py: 42 passed in 39.49 s (includes test_stacking_uses_five_models_and_logistic_regression). Deployed artifact (run_3/stacking.joblib, SHA-256 9c9f0fb1...): pipeline preprocessor -&gt; StackingClassifier with fitted RandomForestClassifier, GradientBoostingClassifier, AdaBoostClassifier, KNeighborsClassifier, GaussianNB; final estimator LogisticRegression; cv 5, predict_proba stacking. End-to-end path to alert shown by TC-02 (alert #2319).</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>test-results/int01_20261019_161543/pytest-int01-units.log, inspect_stacking_modelA.log, inspect_stacking.py; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:03</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>INT-01</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>One byte changed in the cached artifact (local copy, backed up); app restarted: SHA-256 mismatch reported; model not loaded.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>App stopped 16:58 (outbox 919 synced, 0 pending). Cache backed up to C:\AlgoGuardPilot\TC08-backup-models-20261019 (SHA-256 verified equal). Byte at offset 4,279,323 of 1-9c9f0fb1...joblib changed 0x00 -&gt; 0x01 (SHA-256 now c8f1c7fe..., size unchanged). App restarted 17:00:30, PC A analyst signed in. Predict page: 'No active deployment - The cached model is corrupt. Remove it and retry.'; no form, no prediction possible. Live Monitor: the same message, no capture controls. The app neither deleted nor replaced the file. Dashboard still showed the cloud deployment as 'Deployed' with no local warning (DEF-09, Low).</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>DEF-09</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>test-results/int01_20261019_161543/tc08_corruption.json, TC-08_predict_refused.png, TC-08_live_monitor_refused.png, TC-08_dashboard_while_corrupt.png, tc08_flip_byte.py; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:12</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>INT-01</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>After restoring the backup, the app loads the model again (Master Prompt Phase 5.3).</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>App stopped; backup copied back at 17:07; cached file SHA-256 9c9f0fb1...847c again (8,558,646 bytes, only file in the cache). App restarted as administrator, PC A analyst signed in. Predict form shown again; Run Prediction: green verdict at 50.46% confidence, Stacking Ensemble, Deployment #1, latency 2,021.727 ms (first prediction after start), event 3f69afc9..., synced as prediction #3190, no alert. The confidence differs from TC-01 (84.11%): the screenshot shows sinpkt typed as 133.42319, but offline re-scoring of the exact row and of that variant both give Normal 84.11%, so another typed value (not visible, and cleared from the outbox after sync) probably differed. Not counted as a defect; the model loaded and classified.</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>test-results/int01_20261019_161543/TC-08_after_restore_prediction.png, tc08_recheck_row.py, tc08_recheck_row.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:21</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>INT-01</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>CSV replay running in cloud mode; disconnect, restart, reconnect, sign in: pending events kept and synced once; no duplicates.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Baseline 17:15: outbox 920 synced, 0 pending. Live Monitor replay (algoguard_big, Fast, Sequential, Save every flow) started; Wi-Fi switched off (not Airplane mode). Offline: new flows marked Pending; side panel Queued 142, Synced 39, Pending 103, Not stored 0, Upload status 'retrying (transient)'. Capture stopped and app closed offline; app restarted offline: sign-in refused with 'The cloud is unreachable. Online sign-in is required; a cached model does not permit offline access.' (by design); a page showed 'The cloud is unavailable. Pending records stay on this computer.' Wi-Fi on, signed in: Dashboard 17:21 showed Pending 63 durable, Synced 417, Rejected 0, Not stored 0. Outbox 17:21:28: capture session 4ea6f1f9 holds 202 events (17:17:43-17:19:28), all synced, 0 pending; outbox total 1,122 = 920 + 202. 202 distinct event UUIDs and 202 distinct cloud prediction ids, contiguous #3191-#3392; 145 distinct alert ids. No duplicates, none lost.</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>test-results/int01_20261019_161543/TC-09_*.png (sign-in screenshot e-mail redacted), tc09_outbox_check.json, tc09_outbox_sessions.txt; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:24</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01.2</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>CSRF: missing or forged tokens refused; sign-in throttle logic (SEC-01 card; Master Prompt: pytest tests/test_api_validation.py tests/test_login_throttle.py).</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>25 passed in 31.52 s: invalid JSON bodies rejected before any action (16 cases), JSON actions require a JSON content type (2), invalid or forged login tokens return a client error (3); throttle: repeated failures pause the account then release it, success clears the counter, one address cannot spray many usernames, old failures are forgotten. Cookie writes without a CSRF token are also covered by tests/test_cloud_app.py::test_cookie_writes_require_csrf_but_bearer_api_calls_do_not, which passed in TC-13.</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sec01_20261019_172340/pytest-csrf-throttle.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:31</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01.3</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Bandit run; every Medium/High finding fixed or justified, or a defect raised (SEC-01 card; Master Prompt Phase 6).</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Bandit (13:28 scan) by severity: High 0, Medium 14, Low 18. All 14 Medium findings read in the source and justified as false positives: 3 x B104 are an outgoing socket bound to an ephemeral port before connect (cloud_connections.py:177, maintenance_connections.py:141) and a host-name list (maintainer_env.py:44) - nothing listens; 11 x B608 build SQL only from fixed table/column lists or '?' placeholders, with every value passed as a parameter (cloud_outbox.py, legacy_backup.py, legacy_import.py, database_service.py). Hardening suggestion (not a defect): call icacls by full path in cloud_outbox.py:55. No defect raised.</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sec01_20261019_172340/bandit_review.md; test-results/suites_20261019_132412/bandit.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:33</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01.4</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Secrets: git ls-files lists only the .env .example files; git grep for sb_secret_ / service_role / JWT-like strings finds nothing outside tests/fixtures (Master Prompt Phase 6).</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Tracked .env files: .env.example and .env.maintainer.example only. git grep (HEAD): 21 hits, 0 JWT-like strings. Outside tests: service_role is the Postgres role name in 14 migration lines, supabase/config.toml:24 (comment) and docs/migration/05b-access.md:606 (prose); scripts/run_test_suites.py:37 is the redaction regex. Tests: test_cloud_schema.py, test_cloud_app.py, test_cloud_repository.py (fixtures). No secret values found; values were not printed.</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
           <t>Session check with values masked (git ls-files, git grep); evidence: product code = 940e082</t>
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:41</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>SYS-03</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Live re-run: analyst A requests node B's alerts in the UI and Data API: no rows returned; no private data in errors.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: second PC not available (ENV-01.10). Covered by the pilot (SYS-03.P1, SYS-03.P2) and by the automated two-node lane, which passed at 13:30: tests/integration/test_two_node_acceptance.py::test_two_independent_nodes_download_and_write_concurrently and tests/integration/test_relational_access.py (4 tests) against the local Supabase stack.</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:41</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>SYS-03</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Live re-run: administrator revokes B; B tries prediction and capture: both refused; Restore re-enables.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: second PC not available (ENV-01.10). Covered by the pilot (SYS-03.P3) and by tests/integration/test_relational_access.py::test_protected_tables_views_and_revocation, which passed at 13:30.</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>test-results/integration_20261019_132933/pytest-integration.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 17:42</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>TC-15</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner, signed in as an analyst, replays algoguard_big.csv, opens an alert, acknowledges and resolves it: alerts raised for attacks; review actions logged; Product Owner accepts.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: awaiting Product Owner. Four scenarios written for her (replay detection, alert review, report from alerts, administrator approves a node member) with Pass/Fail lines and the accept/reject signature.</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>docs/testing/cycle-1/UAT scenarios.md; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J38"/>
+  <autoFilter ref="A1:J54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2370,7 +3146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3111,8 +3887,150 @@
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>DEF-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.P1 / PRF-01</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Pilot limit L2: p95 upload acknowledgement 24.06 s on one live capture (budget &lt;= 5 s)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>From the pilot record (not re-run in cycle 1):
+1. PC B, live capture 6 on 2026-10-10 (Default interface, save attacks, commit 4c9666c).
+2. Measure upload delay as cloud received_at minus client event_time for the stored events.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>p95 upload acknowledgement &lt;= 5 s (pilot acceptance target, 2026-10-08).</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>'p95 24.06 s, max 36.65 s, with 25 events taking 20-30 s+ around 01:12:25-01:12:44Z.' Not reproduced on 2026-10-16 (capture 19 p95 3.44 s, newer code 940e082); the other 11 runs met the budget. 'Cause not identified.' The pilot recorded it as limit L2 rather than re-targeting it.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>4c9666c (PC B, 2026-10-10)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>PC B (LAPTOP-PNL5IIAJ), Wi-Fi, hosted Supabase pilot (Tokyo)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.P2 / PRF-01</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pilot limit L1: sustained &gt;= 20 acknowledged events/s per client not demonstrated; shipped sources are paced below it</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>From the pilot record (not re-run in cycle 1):
+1. Run a CSV replay at Fast speed and count acknowledged events per second.
+2. Note the replay pace (SPEED_CHOICES: Fast = one flow per 0.35 s) and the 300-event storage cap per capture.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Sustained acknowledged events per client &gt;= 20 events/s (pilot budget; also Master Test Plan 3.4).</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>PC A '≈ 1.9/s (capture 5: 300 events in 157 s)'; PC B 'backlog drain of 210 events in 4.1 s ≈ 51/s'. 'Sources are paced by design: CSV Fast emits one flow per 0.35 s, ≤ 2.9/s. Each capture stores at most 300 events.' 'A sustained-load harness is needed.' Recorded by the pilot as limit L1.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>pilot 4c9666c / 9e18f30</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>PC A and PC B, hosted Supabase pilot (Tokyo)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O10"/>
+  <autoFilter ref="A1:O12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3182,7 +4100,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3214,7 +4132,7 @@
           <t>cb3bcdb</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3246,7 +4164,7 @@
           <t>cb3bcdb</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3278,7 +4196,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3310,7 +4228,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3342,7 +4260,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3374,7 +4292,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3406,7 +4324,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -3438,7 +4356,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3470,7 +4388,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -3502,7 +4420,7 @@
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3579,7 +4497,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3602,7 +4520,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3625,7 +4543,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3652,7 +4570,7 @@
           <t>81.47% (53,243 rows; model A, deployment #1)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -3679,7 +4597,7 @@
           <t>79.49%</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -3706,7 +4624,7 @@
           <t>92.44%</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -3733,7 +4651,7 @@
           <t>25.49%</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -3760,7 +4678,7 @@
           <t>0.9371</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -3783,7 +4701,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3806,7 +4724,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3829,7 +4747,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3852,7 +4770,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3875,7 +4793,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3898,7 +4816,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3921,7 +4839,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -3944,7 +4862,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
         </is>
@@ -4190,19 +5108,19 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -4217,16 +5135,16 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -4253,7 +5171,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
test: record open High defects against the exit criteria
Exit Criteria sheet: 4 High defects open (DEF-04 to DEF-07), so the
'zero open Critical or High' criterion is not met at this point.
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -4542,10 +4542,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>4 High open (DEF-04, DEF-05, DEF-06, DEF-07); 0 Critical (as of 2026-10-19 17:45)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
test: record test cycle 1 results
Final Test Log v1.0: 68 executions (45 pass, 11 fail, 12 not executed),
15 defects (DEF-01 to DEF-15), every exit criterion evaluated, and the
final Testing Kanban snapshot and sync logs.
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,9 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Owner'!$A$1:$G$10</definedName>
   </definedNames>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3134,8 +3134,748 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:51</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>ENV-01.11</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>ENV-01</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>App starts in local (SQLite) mode (ENV-01 card).</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>ALGOGUARD_DB_MODE=sqlite and ALGOGUARD_PORT=5001 set for that process only (.env untouched); python app.py served http://127.0.0.1:5001; /login -&gt; HTTP 200 'Login | AlgoGuard', heading 'Local Console Access' with a username field. Port 5001 was used so the cloud-mode app on 5000 kept running.</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Session check of the local /login page; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:51</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Local mode, account exists: five wrong passwords for one account -&gt; further attempts paused.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Against the local-mode app on port 5001, account 'admin' (the only local account), six sign-ins with made-up wrong passwords sent by script: attempts 1-5 HTTP 200 'Invalid username or password.'; attempt 6 HTTP 429 'Too many failed sign-in attempts. Try again in 15 minutes.' Local system_log: five login_failed (log 115-119) and login_throttled 'Sign-in for admin blocked for 15 minutes after repeated failures.' (log 120), 20:51:21-20:51:23 UTC. The app does not check the password while locked (app.py:398-406), so a correct password would get the same reply; that was not demonstrated because no real password was used. The local app was stopped afterwards, which clears the in-memory lockout. Deviation: the existing admin account was used instead of a throwaway account created on the Admins page.</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sec01_20261019_172340/tc10_lockout.py, tc10_lockout_result.log, tc10_local_db_events.txt; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:52</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01.5</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Analyst role cannot reach administrator pages: signed in as an analyst, /admins and /nodes refused (SEC-01 card; Master Prompt Phase 6).</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Local mode (port 5001): throwaway Analyst 'cycle1_roles_test' created in the local SQLite database with a random password held only in memory; signed in -&gt; Dashboard. GET /admins -&gt; HTTP 302 to / with 'Only Administrator accounts can manage admin users.'; GET /nodes -&gt; 404 (Nodes exists only in cloud mode). (/dashboard -&gt; 404 is a wrong path in the check script; the Dashboard is /.) Cloud mode with a real analyst was not checked by hand; it is covered by tests/test_cloud_app.py::test_administrator_account_management_uses_the_checked_function (a demoted administrator gets 302 from /admins and loses the Accounts link) and the integration tests test_a_token_claiming_administrator_is_not_an_administrator and test_a_profile_cannot_grant_itself_a_role, which passed on 2026-10-19. The local account cycle1_roles_test remains (the app has no delete function).</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sec01_20261019_172340/roles_check.py, roles_check_result.json; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:54</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>POST /predict (and Manual Prediction) with a missing field, text in a numeric field, an out-of-range number: rejected with a plain message; nothing stored.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Server side, through services.simulation_service.predict_with_artifact (used by app.py /simulation and /predict and cloud_app.py:416) with model A, starting from the TC-01 row (control: Normal 84.11%): missing dur -&gt; ACCEPTED, filled with the training default, Normal 56.67%; empty dur -&gt; ACCEPTED, 56.67%; spkts 'abc' -&gt; REJECTED 'spkts must contain a finite numerical value.'; sbytes '1e308' -&gt; REJECTED but with 'Prediction failed: Input X contains infinity or a value too large for dtype('float32').'; sbytes '-5' -&gt; ACCEPTED, Normal 86.65%. Accepted input is classified and queued for upload (cloud_app.py:415-418); the cloud form also fills absent fields with defaults (cloud_app.py:608-611). In the browser, the form's required and number-type boxes block a missing value and 'abc', but there are no min/max limits, so '1e308' and '-5' reach the server. The browser part was not run by hand.</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12, DEF-13</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sys02_files/tc05_server_validation.py, tc05_server_validation_result.json; templates/simulation.html; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:55</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic PCAP, persistence All: all flows classified and saved.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Service level, this cycle: captures/cycle1-tc04-sample.pcap (write_sample_pcap, 10 sessions) through PcapReplaySource and predict_with_artifact with model A: 82 packets -&gt; 11 flows, all classified (10 Attack, 1 Normal; end reasons fin, flush) - the same 11 flows the pilot recorded. Saving was not exercised here. Pilot Test B (2026-10-08, 4c9666c) replayed the same PCAP through the Live Monitor on both PCs: '11 | 11 | 11 -&gt; 0 | 0 of 82 packets' stored -&gt; synced.</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sys02_files/sys02_pcap_service_check.py, sys02_pcap_service_check_result.json, sys02_files_manifest.json; docs/migration/05f-pilot.md §3 Test B; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:55</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.1</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Bad files (empty, text, truncated PCAP) rejected without a crash (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Service level (PcapReplaySource): cycle1-bad-empty.pcap refused 'Unable to read the packet capture: No data could be read!'; cycle1-bad-text.pcap refused 'Unable to read the packet capture: Not a supported capture file'; cycle1-bad-truncated.pcap NOT refused - 49 packets read, 7 flows classified, only a console warning 'Pcap: packet has been truncated'. No crash in any case. The Live Monitor messages for these files were not observed by hand.</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>DEF-14</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>test-results/sys02_files/sys02_pcap_service_check_result.json; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.2</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Live Npcap capture classifies flows and saves results; AlgoGuard's own cloud traffic is excluded (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Not executed this cycle on PC A: live capture needs the app run as administrator and a person at the Live Monitor, and no results were received by close. Pilot evidence: PC A capture 10 (2026-10-15, Administrator) 27 flows, 18 stored, '0 of 848 packets' dropped, '329 own cloud packets excluded'; check_capture_exclusion.py on 2026-10-16 'passed: true' on both PCs ('owned flows classified 0; unrelated flows classified 10').</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>docs/migration/05f-pilot.md §3 Test D; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.3</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>300-event persistence cap shown in the UI (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Not executed this cycle: no replay this cycle reached 300 stored events (SMK-01 stored 275, TC-09 202) and no capped replay was run by close. Automated: tests/test_live_monitor.py asserts persisted &lt;= MAX_PERSISTED_PER_SESSION (passed in TC-13). Pilot: captures 4 and 5 stored '300 (cap)' of 5,000 flows each, and an unplanned replay 'classified 571 flows and stored exactly 300'.</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>docs/migration/05f-pilot.md §3 (Test C, incidental cap evidence); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.1</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Sustained events per second, per client &gt;= 20 (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Measured from this cycle's Fast CSV replays on PC A: TC-09 (Save every flow) 202 events queued 17:17:43-17:19:28 = 105 s -&gt; 1.92 events/s; SMK-01 386 flows analysed in about 190 s (stored events 15:31:20-15:34:30) -&gt; about 2.0 flows/s. The CSV source is paced at one flow per 0.35 s (&lt;= 2.86/s), so 20/s cannot be reached with the shipped sources - same cause as pilot limit L1.</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>test-results/int01_20261019_161543/tc09_outbox_sessions.txt; Test Log SMK-01.3; services/live_monitor_service.py SPEED_CHOICES; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Live capture of ordinary browsing: event-to-verdict lag p95 &lt;= 500 ms (excluding flow timeouts).</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: needs a live capture from an elevated app with someone browsing, and no results were received by close. Measurement note: the app stores no flow end time or per-flow lag (local SQLite stamps flows at classification; the outbox clears payloads after upload), so the lag can only be collected from the live /monitor/status feed (detection_lag_ms, end_reason); test-results/prf01/tc11_collect_lag.js was prepared for that. Pilot reference (different budget): average live lag 13.1 s on PC B including the 15 s idle timeout.</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>test-results/prf01/tc11_collect_lag.js; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.2</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Packet drop during live capture &lt;= 1%; 30-minute soak: CPU &lt;= 80%, RAM &lt;= 1 GiB, no steady growth (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Not executed this cycle: both need a live capture / 30-minute replay started from the browser, and no results were received by close (test-results/prf01/soak_sampler.py was prepared and trial-run: idle app 0.7-1.1% CPU, ~259 MB). Pilot reference (different budgets): packet drop 0% on both PCs; CPU peak 24.5% / 6.3%; RAM peak 294 / 108 MB.</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>test-results/prf01/soak_sampler.py; docs/migration/05f-pilot.md §4; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:56</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>TC-12</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Every page at 390 px (and 1366 px): no page-level horizontal scroll; accessibility scan on Login, Live Monitor and Manual Prediction.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Not executed in this log: no results (screenshots, widths, Lighthouse scores) were received by the log keeper. The Testing Kanban shows USE-01 moved to Done with all four boxes ticked by the card's side on 2026-10-19/20; the log and the board disagree until those results are added. Observation from other cases: alert, log and feed times are shown in UTC without saying so, while 'Deployed at' says UTC.</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Testing Kanban USE-01 card (no attached results); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:01</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.1</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run on the release-candidate commit; no new failures (REG-01 card; TC-14 second half).</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Release candidate 503cb9b = product code 940e082 + the accessibility fix for DEF-15 (templates/monitor.html, static/css/style.css), committed 2026-10-19 19:48 from the USE-01 owner's account and pulled to PC A. run_test_suites.py --all: pytest 537 passed / 67 deselected; ruff all checks passed; pyright 0 errors; node 11 pass; integration 65 passed, 2 skipped (Npcap capture tests, terminal not elevated); pip-audit no known vulnerabilities; Bandit High 0 / Medium 14 / Low 18 - the same findings reviewed in SEC-01.3. No new failures.</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/summary.md and step logs; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:03</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit, then the full automated suite: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Only DEF-15 was fixed during the cycle (503cb9b). The fix is present on the release candidate (the Live Monitor feed container now has tabindex="0", role="region", aria-label="Live monitor feed" and a :focus-visible outline) and the full suite passed on it (REG-01.1). The failing case itself - the Lighthouse accessibility audit of the signed-in Live Monitor page - was not re-run: it needs a signed-in browser and no Lighthouse report was received. DEF-15 stays 'Fixed, re-test pending'. No other defect was fixed in cycle 1.</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>git show 503cb9b; test-results/suites_20261020_045724/; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:03</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: needs a person at the app (sign-in, Manual Prediction, CSV replay) and was not done by close. The change since SMK-01 touches only the Live Monitor feed's markup and CSS; prediction and storage code are unchanged and the full suite passed on 503cb9b.</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>git diff 940e082 503cb9b</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J54"/>
+  <autoFilter ref="A1:J69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3146,7 +3886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4029,8 +4769,296 @@
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TC-05 / SYS-02</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Manual Prediction and /predict accept missing, empty and negative numeric input: missing values are filled with training defaults and the record is saved</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>1. Signed in, POST /predict (JSON) with the TC-01 Normal row but without 'dur', or with 'dur': ''.
+2. Repeat with 'sbytes': '-5'.
+(Equivalent: call services.simulation_service.predict_with_artifact with model A, test-results/sys02_files/tc05_server_validation.py.)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Missing or empty fields and negative byte or packet counts are rejected with a plain message; nothing is classified or stored (TC-05).</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Missing dur -&gt; accepted, filled from the artifact's feature_defaults (simulation_service.py:94), Normal 56.67%; empty dur -&gt; accepted (NaN imputed), 56.67%; sbytes -5 -&gt; accepted, Normal 86.65%. Accepted input is queued for upload (cloud_app.py:415-418). The cloud Manual Prediction form also fills absent fields with defaults before validating (cloud_app.py:608-611). The browser form blocks empty fields (required) but has no min/max, so negatives pass.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5 (product code = 940e082)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; model A (deployment #1)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>DEF-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TC-05 / SYS-02</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>An out-of-range number (1e308) is refused with a technical scikit-learn message, not plain language</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>POST /predict or Manual Prediction with the TC-01 row and sbytes = 1e308.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>A plain message such as 'sbytes is out of range'.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>'Prediction failed: Input X contains infinity or a value too large for dtype('float32').' The value passes the finite-number check (simulation_service.py:99-108) and fails inside the model.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5 (product code = 940e082)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; model A</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>DEF-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.1 / SYS-02</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>A truncated PCAP is replayed partially without telling the user it is cut short</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>1. Use captures/cycle1-bad-truncated.pcap (first 60% of the TC-04 sample).
+2. Replay it (Live Monitor &gt; Recorded packets, or PcapReplaySource directly).</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>The file is rejected, or the user is told the capture is truncated (SYS-02 card: bad files rejected without a crash).</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Not refused: 49 packets read, 7 flows classified; the only sign is a scapy console warning 'Pcap: packet has been truncated'. No crash. Empty and text files are refused correctly.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>dafe5e5 (product code = 940e082)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>TC-12 / USE-01</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Live Monitor's scrolling flow feed cannot be reached by keyboard (Lighthouse: scrollable content not keyboard-accessible)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>1. Sign in and open Live Monitor.
+2. Run Chrome Lighthouse &gt; Accessibility, or press Tab through the page.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Every scrollable region can be focused and scrolled with the keyboard.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Reported through the fix commit 503cb9b ('fix the Ensure elements that have scrollable content are accessible by keyboard in Safari', 2026-10-19 19:48, from the USE-01 owner's account): the .monitor-feed-scroll container had no tabindex, role or label. The Lighthouse report itself was not received by the log keeper.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>940e082 (found); fixed in 503cb9b</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; Chrome Lighthouse</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Fixed - re-test pending</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 REG-01: fix present on 503cb9b (tabindex="0", role="region", aria-label, :focus-visible outline); full suite passed; Lighthouse re-run not executed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O12"/>
+  <autoFilter ref="A1:O16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4041,7 +5069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4407,37 +5435,261 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>2026-10-20 04:59</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pytest-offline: python -m pytest -q</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>537 passed, 67 deselected in 139.19s (0:02:19)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/pytest-offline.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:59</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 ruff-lint: python -m ruff check .</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>All checks passed!</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/ruff-lint.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:00</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pyright-typecheck: npm run typecheck</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>0 errors, 0 warnings, 0 informations</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/pyright-typecheck.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:00</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 node-monitor-poll: node --test tests/monitor_poll.test.cjs</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t># pass 11 / # fail 0</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/node-monitor-poll.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:00</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pytest-integration: python -m pytest -q -m integration</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>65 passed, 2 skipped, 537 deselected in 49.47s</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/pytest-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pip-audit: python -m pip_audit -r requirements.txt</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>No known vulnerabilities found</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/pip-audit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 05:01</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 bandit</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Exit 1 (issues found). By severity: High 0, Medium 14, Low 18 - unchanged, all Medium justified in SEC-01.3. (Runner summary shows the by-confidence counts.)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_045724/bandit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>2026-10-19 13:30</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>pytest-integration re-run after docker start supabase_edge_runtime_AlgoGuard: python -m pytest -q -m integration -rfEs</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>dafe5e5</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>65 passed, 2 skipped, 537 deselected in 43.70s; skips = 2 Npcap capture tests (RUN_WINDOWS_CAPTURE_TESTS not set)</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>test-results/integration_20261019_132933/pytest-integration.log</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4496,15 +5748,19 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>6 of 7 (86%): TC-01, TC-02, TC-03, TC-04, TC-08, TC-09 executed; TC-06 not executed (second PC unavailable - pilot evidence and the automated two-node test only). Counted by card priority instead (Critical cards SMK-01, SYS-01, SYS-03, UAT-01: TC-01, TC-02, TC-03, TC-06, TC-07, TC-15): 3 of 6.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Critical = test cases traced to Critical features F2, F7, F8 in the RTM: TC-01, TC-02, TC-03, TC-04, TC-06, TC-08, TC-09</t>
+          <t>Critical = test cases traced to Critical features F2, F7, F8 in the RTM: TC-01, TC-02, TC-03, TC-04, TC-06, TC-08, TC-09; Test Log</t>
         </is>
       </c>
     </row>
@@ -4519,10 +5775,14 @@
           <t>&gt;= 95%</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>80% of executed test cases (8 of 10: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-13, TC-16 passed; TC-03 and TC-05 failed; TC-06, TC-07, TC-11, TC-12, TC-14, TC-15 not executed). 80.4% of executed Test Log rows (45 Pass of 56).</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4544,7 +5804,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4 High open (DEF-04, DEF-05, DEF-06, DEF-07); 0 Critical (as of 2026-10-19 17:45)</t>
+          <t>4 High open (DEF-04, DEF-05, DEF-06, DEF-07); 0 Critical</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4704,15 +5964,19 @@
           <t>All met or waived</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Events per second not met (about 1.9/s, DEF-11); lag, packet drop and soak not measured this cycle; no written waiver</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>PRF-01 rows below</t>
+          <t>3.4 rows below</t>
         </is>
       </c>
     </row>
@@ -4727,15 +5991,19 @@
           <t>All</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>11 Low/Medium defects open (DEF-01, 02, 03, 08, 09, 10, 11, 12, 13, 14, 15). A workaround is written only in DEF-02 (docker start the Edge Runtime) and DEF-08 (train on 15-feature CSVs); suggested workarounds are in the Completion Report; no Product Owner sign-off yet</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Defects sheet</t>
+          <t>Defects sheet; docs/testing/cycle-1/defects.md</t>
         </is>
       </c>
     </row>
@@ -4750,15 +6018,19 @@
           <t>Generated and accepted</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Generated 2026-10-20 (v1.0); not yet accepted - approval signatures blank</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>DOC-06</t>
+          <t>docs/testing/cycle-1/3 - AlgoGuard Test Completion Report v1.0.docx</t>
         </is>
       </c>
     </row>
@@ -4773,7 +6045,11 @@
           <t>&lt;= 500 ms</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Not measured: TC-11 not executed. The app stores no flow end time or per-flow lag. (Pilot, different budget: average 13.1 s on PC B including the 15 s idle timeout.)</t>
+        </is>
+      </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
@@ -4781,7 +6057,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>PRF-01 / TC-11</t>
+          <t>PRF-01 / TC-11; PRF-01.P3</t>
         </is>
       </c>
     </row>
@@ -4796,15 +6072,19 @@
           <t>&gt;= 20</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>1.92 events/s (TC-09 replay, 202 events in 105 s); about 2.0 flows/s (SMK-01 replay); paced source, max 2.86/s</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>PRF-01.1 · DEF-11</t>
         </is>
       </c>
     </row>
@@ -4819,7 +6099,11 @@
           <t>&lt;= 1%</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Not measured this cycle (pilot: 0% - 0 of 848, 0 of 2,810, 0 of 119,100, 0 of 740 packets)</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
@@ -4827,7 +6111,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>PRF-01.2; PRF-01.P4</t>
         </is>
       </c>
     </row>
@@ -4842,7 +6126,11 @@
           <t>&lt;= 80%</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Not measured this cycle (pilot, different budget: peak 24.5% PC A, 6.3% PC B)</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
@@ -4850,7 +6138,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>PRF-01 soak</t>
+          <t>PRF-01.2; PRF-01.P5</t>
         </is>
       </c>
     </row>
@@ -4865,7 +6153,11 @@
           <t>&lt;= 1 GiB</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Not measured this cycle (pilot: peak 294 MB PC A, 108 MB PC B)</t>
+        </is>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Not measured</t>
@@ -4873,7 +6165,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>PRF-01 soak</t>
+          <t>PRF-01.2; PRF-01.P6</t>
         </is>
       </c>
     </row>
@@ -5031,19 +6323,19 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -5067,10 +6359,10 @@
         <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -5085,10 +6377,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -5112,16 +6404,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>14</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>6</v>
@@ -5139,16 +6431,16 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
test: record the soak, the defect fixes and their re-tests in the test log
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$69</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Owner'!$A$1:$G$10</definedName>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Not executed: awaiting Product Owner. Four scenarios written for her (replay detection, alert review, report from alerts, administrator approves a node member) with Pass/Fail lines and the accept/reject signature.</t>
+          <t>Not executed: awaiting Product Owner. Four scenarios written for her (replay detection, alert review, report from alerts, administrator approves a node member) with Pass/Fail lines and the accept/reject signature. On 2026-10-20 the Lead Architect relayed that she gave permission to accept the build; no executed scenarios or signed decision were received.</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -3874,8 +3874,1304 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:06</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>App restarted as administrator on 503cb9b; PC A analyst signed in once in a test Chrome window driven by script (Playwright over CDP). TC-01 Normal row -&gt; NORMAL 84.11%, deployment #1, synced as prediction #4160, no alert. TC-02 Attack row -&gt; ATTACK 92.95%, synced as prediction #4161 with alert #3369. Short replay (algoguard_big, Fast, Save attacks, 120 s): 172 flows, 126 Attack / 46 Normal, 126 alerts, 126 queued, 126 synced, 0 pending, 0 not stored, no error. Two earlier attempts at 05:53-05:54 failed on a screenshot step after submitting; their 3 manual predictions were synced and are extra records, not results.</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/smk_rerun.json, smk_*.png, outbox_sessions_0600.txt; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:08</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Malformed input on Manual Prediction: missing field, text in a numeric field, an out-of-range number, a negative byte count - rejected with a plain message; nothing stored.</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Real form, starting from the TC-01 row: (a) dur emptied -&gt; browser blocks the submit, 'Please fill out this field.'; (b) typing 'abc' into spkts leaves it empty -&gt; 'Please fill out this field.'; (c) sbytes 1e308 -&gt; 'Prediction failed: Input X contains infinity or a value too large for dtype('float32').' (DEF-13); (d) sbytes -5 -&gt; ACCEPTED, NORMAL 86.65%, event cb1438e0, stored and synced as prediction #4288 (DEF-12). (a) and (b) are stopped only by the browser; the server accepts them (TC-05 at 04:54).</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12, DEF-13</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/sys02_ui.json, tc05_*.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:08</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic PCAP, persistence All: all flows classified and saved.</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Live Monitor, Recorded packets (PCAP), cycle1-tc04-sample.pcap, Fast, Save every flow: 11 of 11 flows, 10 Attack / 1 Normal, 10 alerts, 11 queued, 11 synced, 0 pending, 0 not stored; 'The traffic source finished streaming.'</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/sys02_ui.json, pcap_cycle1-tc04-sample.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:08</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.1</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Bad files (empty, text, truncated PCAP) rejected without a crash (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Live Monitor: cycle1-bad-empty.pcap -&gt; 'Unable to read the packet capture: No data could be read!'; cycle1-bad-text.pcap -&gt; 'Unable to read the packet capture: Not a supported capture file'; cycle1-bad-truncated.pcap -&gt; 7 of 7 flows streamed and saved, 'The traffic source finished streaming.', no warning (DEF-14). No crash; the page kept working.</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>DEF-14</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/sys02_ui.json, pcap_*.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:15</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.3</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>300-event persistence cap shown in the UI (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Sample replay algoguard_big, Fast, Save every flow: side panel 'Queued for upload 300 (capped)', 'Not stored 312', classification continued to 612 flows (438 Attack); 211 alerts; Synced 300, Pending 0. Outbox: session 749511b1 holds exactly 300 events, all synced, 211 with alerts. The cap is shown in the Queued-for-upload field; no separate message.</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/sys02_ui.json, cap_300.png, outbox_sessions_0600.txt; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:19</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>TC-12</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Every page at 390 px (and 1366 px): no page-level horizontal scroll.</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard, Live Monitor, Manual Prediction, Alerts, System Logs, Reports, Nodes, Accounts/Admins and Login at 1366x768 and 390x844 (fresh tab, signed-in session): document scrollWidth never above the window width (375-390 of 390; 1351-1366 of 1366), no element outside a scroll container past the right edge; screenshots show stacked layouts with no overlap. Accounts/Admins redirects the analyst to the Dashboard.</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/use01/use01_ui.json and 18 screenshots; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:19</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.1</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard navigation and form labels checked on Login, Live Monitor and Manual Prediction (USE-01 card).</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Tab walk: Login 3 of 3 interactive elements reached, Live Monitor 17 of 17, Manual Prediction 25 of 25 distinct (26 counting a second 'Live Monitor' link); no visible field without a label (label element, aria-label or aria-labelledby).</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/use01/use01_ui.json; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:23</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.2</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Automated accessibility scan run; serious issues logged as DEF cards (USE-01 card).</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Lighthouse 12.6.0, desktop, Accessibility only: Login 100 (signed-out Chrome), Live Monitor 100 and Manual Prediction 100 (signed-in session, storage reset disabled); 0 failed audits on each.</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/lighthouse/ (reports and lighthouse_summary.json); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:24</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15 re-test on 503cb9b: the Live Monitor feed has tabindex=0, role=region, aria-label 'Live monitor feed'; reached with Tab (17th stop); PageDown scrolled it from 0 to 420 px of 2,084 px content; visible focus outline (solid 1.6px). Lighthouse 12.6 has no scrollable-region audit, so the behaviour was tested directly. Full suite passed on 503cb9b (REG-01.1). DEF-15 closed.</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/def15_check.json, def15_feed_focused.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:26</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.2</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Live Npcap capture classifies flows and saves results; AlgoGuard's own cloud traffic is excluded (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Live interface capture, default interface, Save attacks, 06:24:38-06:26:08 (90 s) while about 100 public web pages were fetched: 8,721 packets, 0 dropped, 1,025 own cloud packets excluded; 139 flows classified (93 Attack / 46 Normal; ended by FIN 14, RST 18, idle timeout 107); 93 saved, 93 synced, 0 pending. Observation: 67% of ordinary browsing flagged Attack - same pattern as pilot finding 12 and consistent with DEF-06.</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/tc11_live.json, live_capture.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:26</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Live capture of ordinary browsing: event-to-verdict lag p95 &lt;= 500 ms (excluding flow timeouts).</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Same 90 s capture. Lag per flow read from the page's /monitor/status feed (detection_lag_ms = verdict time minus the flow's last packet). Flows ended by TCP FIN/RST (no timeout wait), n=32: p50 388.9 ms, p95 895.6 ms - budget missed. All 139 flows: p50 15,765 ms, p95 16,311 ms (includes the 15 s idle timeout); idle-timeout flows minus 15 s: p50 916.5 ms, p95 1,362.4 ms. Model latency: p50 163.9 ms, p95 377.2 ms. A traffic generator and Chrome were running on PC A.</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/tc11_live.json; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:26</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.3</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Packet drop fraction during live capture &lt;= 1% (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>0 of 8,721 packets dropped (0%) in the 90 s live capture.</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/tc11_live.json (session_capture_counters); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:27</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Error messages and status text are plain language (USE-01 card).</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Mostly plain (e.g. 'Unable to read the packet capture: Not a supported capture file', 'Please fill out this field.'). Not plain: the 1e308 message 'Input X contains infinity or a value too large for dtype('float32')' (DEF-13); System Logs show the word 'None' as the message of every flow_accepted entry (DEF-18); feed, alert and log times are UTC without a label - the newest log line reads 2026-10-19 22:15:46 for 2026-10-20 06:15:46 local (DEF-16).</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>DEF-13, DEF-16, DEF-18</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/use01/1366_logs.png, use01/390_monitor.png, tc05_c_1e308.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:57</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.4</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>30-minute soak: AlgoGuard process CPU &lt;= 80% and RAM &lt;= 1 GiB, no steady growth (plan 3.4; PRF-01 card).</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Live Monitor, Sample replay algoguard_biggest.csv, Fast, Sequential, Save attacks, 06:27:23-06:57:25 (1,800 s), started and stopped by script in the signed-in test Chrome. Sampler every 30 s on the app (PID 37452 + its 3.5 MB launcher, found by command line), 60 samples 06:28:02-06:57:33. CPU (share of the whole machine): max 8.03%, mean 7.54%. RAM: max 352.2 MB (first 4 minutes), dropped to 298.6 MB at 06:32, climbed to 327.8 MB by 06:55 (about 1.1 MB/min), flat from 06:52 (+1 MB), 322.0 MB at the end; whole-run trend -0.1 MB/min. Threads 35-37. No error message; 300 stored (cap), 300 synced, 0 pending. Observation: 30 minutes cannot rule out a slow leak after the 06:32-06:52 climb; a longer soak is suggested for cycle 2. Short test runs in other processes ran on PC A during the soak.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>test-results/soak_20261020_062732.csv; test-results/ui_20261020/soak_ui.json, soak_sampler_console.log, soak_end.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:57</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.5</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Sustained events per second, per client &gt;= 20 (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Same 30-minute Fast replay: 2,972 flows classified in 1,800 s = 1.65 flows/s (five-minute readings 498, 1,025, 1,548, 2,043, 2,477, 2,972); 300 events stored (the per-session cap), all synced. The sample source is paced at one flow per 0.35 s (&lt;= 2.86/s), so 20/s cannot be reached with it.</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/soak_ui.json, soak_end.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:01</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>DEF-09 (fixed in eecaac7 and 0480899) re-tested with the TC-08 procedure on a backed-up cache: cache file 1-9c9f0fb185... (8,558,646 bytes) copied to C:\AlgoGuardPilot\REG01-backup-models-20261020 (SHA-256 checked), one byte changed at offset 4,279,323; app restarted on 0480899 and the PC A analyst signed in. Dashboard: model label 'Unavailable here' and 'Not usable on this computer: The cached model is corrupt. Remove it and retry.'; Manual Prediction: 'No active deployment - The cached model is corrupt. Remove it and retry.' Cache restored from the backup at 07:01:18 (SHA-256 matches again), no restart needed: Dashboard 'Deployed', Manual Prediction form back with 15 fields. DEF-09 closed.</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>DEF-09</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/def09_check.json, def09_dashboard_corrupt.png, def09_dashboard_restored.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Malformed input on Manual Prediction: missing field, text in a numeric field, an out-of-range number, a negative byte count - rejected with a plain message; nothing stored.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Re-run of (c) and (d) on the fix build, signed-in test Chrome, starting from the TC-01 row: (c) sbytes 1e308 -&gt; 'sbytes is too large to classify; enter a smaller value.'; (d) sbytes -5 -&gt; browser: 'Value must be greater than or equal to 0.'; the same form with the browser check off -&gt; 'sbytes cannot be negative.'; /predict with sbytes -5, dur -1 and sbytes 1e308 -&gt; HTTP 400 with the same plain messages. Flows Analyzed 2,277 before and after: nothing stored. (a) and (b) not re-run (browser-blocked at 06:08; unchanged). Still failing: a missing or empty numeric field sent to the server is filled with the training default and stored - unchanged design, asserted by test_missing_numeric_prediction_is_imputed_and_saved_as_null, which passed on this build (REG-01.1).</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (tc05), tc05_*.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02.1</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Bad files (empty, text, truncated PCAP) rejected without a crash (SYS-02 card).</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Live Monitor, Recorded packets, Save every flow: cycle1-bad-truncated.pcap -&gt; 'The packet capture is incomplete: its last packet is cut off. Use a complete capture file.', 0 flows, nothing stored, page kept working. Empty and text files not re-run (refused without a crash at 06:08).</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>DEF-14</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (pcap), pcap_cycle1-bad-truncated.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic PCAP, persistence All: all flows classified and saved.</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Regression re-run after the PCAP change: cycle1-tc04-sample.pcap, Fast, Save every flow: 11 of 11 flows, 10 Attack / 1 Normal, 10 alerts, 11 queued, 11 synced, 0 pending, 0 not stored; 'The traffic source finished streaming.'</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (pcap), pcap_cycle1-tc04-sample.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Error messages and status text are plain language (USE-01 card).</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Fix build: Logs header 'Timestamp (UTC)', Alerts 'Detected (UTC)', Live Monitor 'Time (UTC)', Dashboard alert and log lines end in 'UTC' (7); 0 of 21 flow_accepted rows show 'None' (DEF-18 fixed); the 1e308 message is plain (TC-05 at 07:02). Still unlabelled UTC times: Dashboard 'Last at 2026-10-19 22:31:50' under Flows Analyzed, Nodes 'Requested'/'Decided', Accounts 'Created' and local-mode 'Deployed at' (DEF-16 not fully fixed; follow-up fix 128855e).</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>DEF-16</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (labels), def09_dashboard_corrupt.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:03</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.1</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run on the fix build; no new failures (REG-01 card; TC-14 second half).</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Fix build 0480899 = 503cb9b + eight fix commits for DEF-01, 02, 03, 08, 09, 12, 13, 14, 16 and 18 (eecaac7..0480899). run_test_suites.py --all 06:58-07:03: pytest 550 passed / 67 deselected (13 more than on 503cb9b, the new tests for the fixes); pyright 0 errors; node 11 pass; integration 65 passed, 2 skipped (Npcap capture tests, terminal not elevated); pip-audit no known vulnerabilities; Bandit High 0 / Medium 14 / Low 18 (same as SEC-01.3). Ruff found 3 over-long lines, all in an uncommitted evidence script (test-results/ui_20261020/lighthouse/summarise_lighthouse.py), none in product code; after re-wrapping it (its output is unchanged) ruff check . passed. No new failures in product code.</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_065849/summary.md and step logs; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:03</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01.4</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>SEC-01</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Arella Biacea B. Mirasol</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>No secrets in pages or API responses (SEC-01 card).</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Signed-in analyst session, same-session requests to /, /monitor, /monitor/status, /simulation, /alerts, /logs, /reports, /nodes, /admins (redirects an analyst to the Dashboard) and /outbox/export: all HTTP 200, 0 matches for JWTs, Supabase keys, 'service_role', Bearer tokens, password/secret/key/token values, SUPABASE_/ALGOGUARD_ setting names and e-mail addresses (counts only were saved). No report existed to open, so report detail pages were not scanned. Repository and logs were checked in SEC-01 on 2026-10-19. Note: a UTC label edit to the Nodes page template was briefly on disk in the repository folder around 07:02-07:03 and then undone, so the Nodes header text may have come from it (label text only; no effect on this scan).</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (secrets); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:05</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the fix build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>TC-01 Normal row -&gt; NORMAL 84.11%, deployment #1, synced as prediction #5011, no alert. TC-02 Attack row -&gt; ATTACK 92.95%, synced as prediction #5012 with alert #4126. Replay algoguard_big, Fast, Save attacks, 07:03:24-07:05:24: 167 flows, 121 Attack / 46 Normal, 121 alerts, 121 queued, 121 synced, 0 pending, 0 not stored, no error. Outbox: all 2,099 events synced.</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/reg01_ui.json (smoke), smk_*.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:05</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>DEF-13 (edf6193): 1e308 now refused in plain language at the form and /predict - closed. DEF-12 (edf6193): negative values now refused at the browser, the form and /predict, nothing stored; missing or empty numeric fields are still filled with training defaults and stored at the server (deliberate design, not changed) - TC-05 still fails on that part; DEF-12 stays open for a decision. DEF-14 (547044f): truncated capture refused, TC-04 sample unaffected - closed. DEF-18 (1ffa1b9): no 'None' messages - closed. DEF-16 (1ffa1b9): partly fixed; remaining labels in 128855e, re-tested on the final build.</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12, DEF-13, DEF-14, DEF-16, DEF-18</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Test Log rows TC-05, SYS-02.1, TC-04, USE-01.3 at 07:02; test-results/ui_20261020/reg01/; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:09</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.1</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>128855e</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run on the final build; no new failures (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Final build 128855e (0480899 + the remaining UTC labels for DEF-16): pytest 551 passed / 67 deselected; ruff all checks passed; pyright 0 errors; node 11 pass. Integration lane: see INT-01.2.</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_final_128855e/*.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:13</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>128855e</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>DEF-08 (2f4e087): the raw research/dataset/raw/UNSW_NB15_training-set.csv (45 columns incl. id and attack_cat) given to the training preparation on the final build -&gt; 15 training columns, exactly the live flow features; id and attack_cat not used. Training itself was not re-run (no new model or run written). Not changed: local train.py --deploy still has no feature-schema check (local mode allows other schemas by design), so DEF-08 stays open for that part.</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>DEF-08</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/reg01/def08_schema_check.txt; tests/test_training_schema.py; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
+  <autoFilter ref="A1:J95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3886,7 +5182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4552,8 +5848,16 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>2f4e087 (training columns only)</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:13 TC-14 Pass for the reported case: the raw UNSW-NB15 training file now gives exactly the 15 flow features (no id, no attack_cat). Still open: local train.py --deploy has no feature-schema check (local mode allows other schemas by design; needs a decision).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4621,11 +5925,19 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>eecaac7, 0480899</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:01 TC-14 Pass: with a corrupted cached copy the Dashboard shows 'Unavailable here' and the reason; after restoring the backup it shows 'Deployed' again.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4837,8 +6149,16 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>edf6193 (negative values only)</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02 TC-05 re-run: negative values refused at the browser, the form and /predict, nothing stored - Pass for that part. Still open: missing or empty numeric fields are filled with training defaults and stored at the server (deliberate, tested design; needs a decision by the Lead Architect and Product Owner).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4903,11 +6223,19 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>edf6193</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02 TC-05 re-run Pass: 1e308 -&gt; 'sbytes is too large to classify; enter a smaller value.' at the form and /predict; nothing stored.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4973,11 +6301,19 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>547044f</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02 SYS-02.1 re-run Pass: 'The packet capture is incomplete: its last packet is cut off. Use a complete capture file.', 0 flows; TC-04 sample still 11 of 11 flows.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5043,7 +6379,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Fixed - re-test pending</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -5053,12 +6389,230 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 REG-01: fix present on 503cb9b (tabindex="0", role="region", aria-label, :focus-visible outline); full suite passed; Lighthouse re-run not executed.</t>
+          <t>2026-10-20 06:24 TC-14 Pass: feed reached with Tab, PageDown scrolls it, focus outline visible; Lighthouse 12.6 Accessibility 100 on Live Monitor; full suite passed on 503cb9b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DEF-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3 / USE-01</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Feed, alert and log times are shown in UTC without saying so</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>1. On PC A (UTC+8), run a replay at a known local time.
+2. Read the Recent Flows TIME column, the Dashboard alerts and System Logs.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Times in local time, or clearly labelled UTC as 'Deployed at' and Reports ('Generated (UTC)') already are.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Recent Flows shows 22:15:45 for a flow at 06:15:45 local; System Logs' newest line reads 2026-10-19 22:15:46 for 2026-10-20 06:15:46 local - even the date looks a day behind. Seen in SMK-01, TC-09 and USE-01.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; cloud mode</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>TC-11 / PRF-01</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Live event-to-verdict lag p95 is 895.6 ms for flows ended by FIN/RST (budget &lt;= 500 ms)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>1. Start the app as administrator; Live Monitor &gt; Live interface capture, Save attacks.
+2. Browse normally for 90 s.
+3. Read detection_lag_ms and end_reason per flow from /monitor/status; take flows with end_reason fin or rst.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>p95 &lt;= 500 ms (Master Test Plan 3.4).</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>n=32 FIN/RST flows: p50 388.9 ms, p95 895.6 ms. Model latency alone p50 163.9 ms, p95 377.2 ms, so roughly half the delay is queueing and handling around the model. Measured with a traffic generator and Chrome running on PC A; the app also stores no per-flow lag, so this can only be measured live.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; Intel Wi-Fi 6 AX203, Npcap 1.88, administrator</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>DEF-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3 / USE-01</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>System Logs show the word 'None' as the message of every flow_accepted entry</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Run any replay in cloud mode, then open Logs.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>An empty message cell or a readable message.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Each 'detection / flow_accepted / success' row has the message 'None' (a Python null rendered as text).</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>503cb9b</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>PC A (SANMIGUEL), Windows 11 Home 26H2 build 26300.9711, Python 3.14.6 venv; cloud mode</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>1ffa1b9</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02 USE-01.3 re-run: 0 of 21 flow_accepted rows show 'None' - Pass.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O16"/>
+  <autoFilter ref="A1:O19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5777,7 +7331,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>80% of executed test cases (8 of 10: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-13, TC-16 passed; TC-03 and TC-05 failed; TC-06, TC-07, TC-11, TC-12, TC-14, TC-15 not executed). 80.4% of executed Test Log rows (45 Pass of 56).</t>
+          <t>69% of executed test cases (9 of 13: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-12, TC-13, TC-16 passed; TC-03, TC-05, TC-11 and TC-14 failed - TC-14 because the DEF-12 re-test still fails; TC-06, TC-07, TC-15 not executed). 76.8% of executed Test Log rows (63 Pass of 82).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -5966,7 +7520,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Events per second not met (about 1.9/s, DEF-11); lag, packet drop and soak not measured this cycle; no written waiver</t>
+          <t>Lag p95 not met (895.6 ms, DEF-17) and events per second not met (1.65-1.92/s, DEF-11); packet drop, soak CPU and soak RAM met; no written waiver</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -5993,7 +7547,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>11 Low/Medium defects open (DEF-01, 02, 03, 08, 09, 10, 11, 12, 13, 14, 15). A workaround is written only in DEF-02 (docker start the Edge Runtime) and DEF-08 (train on 15-feature CSVs); suggested workarounds are in the Completion Report; no Product Owner sign-off yet</t>
+          <t>9 Low/Medium defects open (DEF-01, 02, 03, 08, 10, 11, 12, 16, 17); DEF-09, 13, 14, 15 and 18 fixed and closed in REG-01. Fix commits for DEF-01/03 (CI) and the rest of DEF-16 wait for their re-test. Workarounds written in DEF-02 (README) and DEF-08 (train on 15-feature CSVs); no Product Owner sign-off yet</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -6047,17 +7601,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Not measured: TC-11 not executed. The app stores no flow end time or per-flow lag. (Pilot, different budget: average 13.1 s on PC B including the 15 s idle timeout.)</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+          <t>895.6 ms p95 (p50 388.9 ms) over 32 flows ended by FIN/RST in a 90 s live capture of ordinary browsing on PC A</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Not met</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>PRF-01 / TC-11; PRF-01.P3</t>
+          <t>TC-11 · test-results/ui_20261020/tc11_live.json · DEF-17</t>
         </is>
       </c>
     </row>
@@ -6074,7 +7628,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1.92 events/s (TC-09 replay, 202 events in 105 s); about 2.0 flows/s (SMK-01 replay); paced source, max 2.86/s</t>
+          <t>1.65 flows/s over the 30-minute Fast replay; 1.92 events/s (TC-09 replay, 202 events in 105 s); paced source, max 2.86/s</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -6084,7 +7638,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.1 · DEF-11</t>
+          <t>PRF-01.5, PRF-01.1 · DEF-11</t>
         </is>
       </c>
     </row>
@@ -6101,17 +7655,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Not measured this cycle (pilot: 0% - 0 of 848, 0 of 2,810, 0 of 119,100, 0 of 740 packets)</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+          <t>0% (0 of 8,721 packets in the 90 s live capture)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.2; PRF-01.P4</t>
+          <t>PRF-01.3 · test-results/ui_20261020/tc11_live.json</t>
         </is>
       </c>
     </row>
@@ -6128,17 +7682,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Not measured this cycle (pilot, different budget: peak 24.5% PC A, 6.3% PC B)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+          <t>Max 8.03%, mean 7.54% of the machine (60 samples, 06:28-06:57)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.2; PRF-01.P5</t>
+          <t>PRF-01.4 · test-results/soak_20261020_062732.csv</t>
         </is>
       </c>
     </row>
@@ -6155,17 +7709,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Not measured this cycle (pilot: peak 294 MB PC A, 108 MB PC B)</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Not measured</t>
+          <t>Max 352.2 MB; 322.0 MB at the end; whole-run trend -0.1 MB/min (a climb of about 29 MB from 06:32 to 06:52 then flat - a longer soak is suggested)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.2; PRF-01.P6</t>
+          <t>PRF-01.4 · test-results/soak_20261020_062732.csv</t>
         </is>
       </c>
     </row>
@@ -6323,13 +7877,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2</v>
@@ -6350,19 +7904,19 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -6377,10 +7931,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -6404,19 +7958,19 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -6431,13 +7985,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
test: record the CI re-test, the final checks and the closed defects in the test log
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5170,8 +5170,212 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:29</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02.1</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>ccbadd8</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Run 39341292642 on ccbadd8 (product code 128855e plus test records), 07:23-07:29: setup-python 'python-version: 3.14.6' -&gt; 'Successfully set up CPython (3.14.6)'; Lint 'All checks passed!'; Type check '0 errors, 26 warnings'; Unit tests '535 passed, 21 skipped, 34 deselected'; Browser polling tests 11 pass / 0 fail; conclusion success - the first green run on main since 2026-10-05.</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>DEF-01, DEF-03</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>test-results/env_20261020/ci_run_39341292642_ccbadd8_success.log; https://github.com/AlgoGuard-CSThesis/AlgoGuard/actions/runs/39341292642; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:29</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>ccbadd8</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>DEF-01 and DEF-03 (f143b21): CI run 39341292642 installs the locked Python 3.14.6, and the model-loading tests and the outbox cap test pass on the runner; all four CI checks green (ENV-02.1 at 07:29) - both closed. DEF-02 (8b5133c): the README now tells testers to check 'Stopped services' after supabase start and restart the Edge Runtime; the integration lane passed with all services up (REG-01.1 at 07:03). The Supabase CLI behaviour itself is outside AlgoGuard - closed with the workaround documented.</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>DEF-01, DEF-02, DEF-03</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>test-results/env_20261020/ci_run_39341292642_ccbadd8_success.log; README.md; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:44</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Every shown time labelled UTC after the follow-up fix 128855e (DEF-16 re-test on the final build).</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Planned on 128855e, but the app on port 5000 was still the process started at 07:00:28 on 0480899 (not restarted after main moved to 128855e), so the 128855e labels were not exercised. Seen on 0480899: Logs, Alerts, Live Monitor and Reports headers say UTC; 0 'None' messages; Dashboard 'Deployed at 2026-10-08 06:10:49 UTC'; still unlabelled: 'Last at 2026-10-19 23:05:24' and the Nodes 'Decided' header - as expected for 0480899. The 128855e labels are covered only by the automated tests that passed on 128855e (REG-01.1 at 07:09).</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>DEF-16</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/final/final_ui.json (labels; screenshots not captured - the browser window could not be drawn); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:47</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>0480899</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Second smoke run, again on the 0480899 process (the app was not restarted on the final build 128855e, whose only product change is UTC label text in four templates). TC-01 -&gt; NORMAL 84.11%, no alert; TC-02 -&gt; ATTACK 92.95%, alert on upload; replay algoguard_big, Fast, Save attacks, 09:44:54-09:46:58: 191 flows, 138 Attack / 53 Normal, 138 alerts, 138 queued, 138 synced, 0 pending, 0 not stored, no error.</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/final/final_ui.json (smoke), smk_replay.png (the TC-01/TC-02 screenshots were not captured); evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J95"/>
+  <autoFilter ref="A1:J99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5345,11 +5549,19 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>f143b21</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:29 ENV-02.1 Pass: CI run 39341292642 sets up CPython 3.14.6; unit tests 535 passed, 21 skipped; all four checks green.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -5416,11 +5628,19 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>8b5133c (README workaround)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:03 integration lane 65 passed, 2 skipped with all services up. The Supabase CLI still exits 0 with a stopped container (outside AlgoGuard); the README step is the documented workaround.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5486,11 +5706,19 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>f143b21</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:29 ENV-02.1 Pass: the outbox cap test passes on the CI runner (run 39341292642).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -6460,8 +6688,16 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>1ffa1b9, 128855e</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:02 USE-01.3 on 0480899: feed, alert, log and report times now say UTC, but Dashboard 'Last at', Nodes, Accounts and local 'Deployed at' did not - fixed in 128855e, whose automated tests passed (07:09). UI re-test on 128855e not executed (app not restarted); stays open until then.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7331,7 +7567,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>69% of executed test cases (9 of 13: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-12, TC-13, TC-16 passed; TC-03, TC-05, TC-11 and TC-14 failed - TC-14 because the DEF-12 re-test still fails; TC-06, TC-07, TC-15 not executed). 76.8% of executed Test Log rows (63 Pass of 82).</t>
+          <t>69% of executed test cases (9 of 13: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-12, TC-13, TC-16 passed; TC-03, TC-05, TC-11 and TC-14 failed - TC-14 because the DEF-12 re-test still fails; TC-06, TC-07, TC-15 not executed). 76.7% of executed Test Log rows (66 Pass of 86).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -7547,7 +7783,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>9 Low/Medium defects open (DEF-01, 02, 03, 08, 10, 11, 12, 16, 17); DEF-09, 13, 14, 15 and 18 fixed and closed in REG-01. Fix commits for DEF-01/03 (CI) and the rest of DEF-16 wait for their re-test. Workarounds written in DEF-02 (README) and DEF-08 (train on 15-feature CSVs); no Product Owner sign-off yet</t>
+          <t>6 Low/Medium defects open (DEF-08, 10, 11, 12, 16, 17); DEF-01, 02, 03, 09, 13, 14, 15 and 18 fixed and closed in REG-01. DEF-08 and DEF-12 are fixed in part and wait for a decision; DEF-16 waits for its UI re-test on 128855e. Workaround written in DEF-08 (train on 15-feature CSVs); no Product Owner sign-off yet</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -7904,13 +8140,13 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
@@ -7958,10 +8194,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>9</v>
@@ -7985,10 +8221,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
test: record the final-build re-tests; DEF-08, DEF-12 and DEF-16 closed
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J99"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5374,8 +5374,408 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:02</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02.1</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>33ca81d</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Run 39356261813 on 33ca81d (final product code 128855e plus test records and reports), 09:57-10:02: 'Successfully set up CPython (3.14.6)'; Lint 'All checks passed!'; Type check '0 errors, 26 warnings'; Unit tests '535 passed, 21 skipped, 34 deselected'; Browser polling tests 11 pass / 0 fail; conclusion success.</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>test-results/env_20261020/ci_run_39356261813_33ca81d_success.log; https://github.com/AlgoGuard-CSThesis/AlgoGuard/actions/runs/39356261813; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:17</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.1</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run on the final build; no new failures (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Final build 213d0be = 128855e + the DEF-12 fix (063f42f) and the DEF-08 fix (213d0be): pytest 566 passed / 67 deselected; ruff all checks passed; pyright 0 errors; node 11 pass; integration 65 passed, 2 skipped (Npcap capture tests, terminal not elevated). No new failures.</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_101708/*.log; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:17</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>DEF-08 (2f4e087, 213d0be): the raw UNSW file trains on exactly the 15 flow features (07:13 check); any training file now loses id and attack_cat, also without the full flow schema and with a byte-order mark (test_id_and_attack_cat_are_never_features_even_without_the_full_flow_schema); train.py names missing and extra columns and says Live Monitor and publishing will refuse such a model (test_live_schema_note_*). Live Monitor already refuses incompatible models before capture. All passed in REG-01.1 at 10:17 - closed.</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>DEF-08</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261020_101708/pytest-offline.log; tests/test_training_schema.py; tests/test_cli_training.py; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:20</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>USE-01.3</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>USE-01</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Brynt M. Timtiman</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Error messages and status text are plain language; every shown time says it is UTC (USE-01 card; DEF-16 re-test on the final build).</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>App restarted at 10:19:41 on the final build 213d0be, analyst signed in. Dashboard 'Last at 2026-10-20 01:46:58 UTC' and 'Deployed at 2026-10-08 06:10:49 UTC' (no doubled 'UTC'), alert and log lines end in UTC (7); headers: Logs 'Timestamp (UTC)', Alerts 'Detected (UTC)', Live Monitor 'Time (UTC)', Reports 'Generated (UTC)', Nodes 'Decided (UTC)'; 0 'None' log messages.</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>DEF-16</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/final2/final2_ui.json (labels), dashboard_utc.png, nodes_utc.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:20</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>SYS-02</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>John Brian A. Tiopes</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Malformed input on Manual Prediction: missing field, text in a numeric field, an out-of-range number, a negative byte count - rejected with a plain message; nothing stored.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Final build: (a) dur emptied in the form with the browser check off -&gt; 'Enter a value for every field; missing: dur.'; /predict with dur omitted, null or empty -&gt; HTTP 400 with the same message. Flows Analyzed 2,551 before and after: nothing stored. (b) 'abc' is blocked by the browser number field (06:08) and refused by the server ('must contain a finite numerical value', unit tests); (c) 1e308 and (d) negative values refused in plain language (07:02, unchanged code). All four inputs are now refused and nothing is stored.</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/final2/final2_ui.json (def12), def12_form_empty_dur.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:23</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02.1</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests) (ENV-02 card).</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Run 39358135540 on the final build 213d0be, finished 10:22:59: 'Successfully set up CPython (3.14.6)'; Lint 'All checks passed!'; Type check '0 errors, 26 warnings'; Unit tests '550 passed, 21 skipped, 34 deselected'; Browser polling tests 11 pass / 0 fail; conclusion success.</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr"/>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>test-results/env_20261020/ci_run_39358135540_213d0be_success.log; https://github.com/AlgoGuard-CSThesis/AlgoGuard/actions/runs/39358135540; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:23</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Final build 213d0be: TC-01 Normal row -&gt; NORMAL 84.11%, deployment #1, synced as prediction #5274, no alert. TC-02 Attack row -&gt; ATTACK 92.95%, synced as prediction #5275 with alert #4387. Replay algoguard_big, Fast, Save attacks, 10:21:22-10:23:22: 169 flows, 123 Attack / 46 Normal, 123 alerts, 123 queued, 123 synced, 0 pending, 0 not stored, no error. Outbox: all 2,364 events synced.</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/final2/final2_ui.json (smoke), smk_*.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:23</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12 (edf6193, 063f42f): TC-05 passes on the final build - omitted, null and empty fields refused at the form and /predict, nothing stored - closed. DEF-16 (1ffa1b9, 128855e): every shown time says UTC on the final build (USE-01.3 at 10:20) - closed. Every fixed DEF card is now re-tested and closed; open: the cycle 2 items DEF-04..07, 10, 11, 17.</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>DEF-12, DEF-16</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Test Log rows TC-05, USE-01.3 and REG-01.2 at 10:20-10:23; test-results/ui_20261020/final2/; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J99"/>
+  <autoFilter ref="A1:J107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6073,17 +6473,17 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2f4e087 (training columns only)</t>
+          <t>2f4e087, 213d0be</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:13 TC-14 Pass for the reported case: the raw UNSW-NB15 training file now gives exactly the 15 flow features (no id, no attack_cat). Still open: local train.py --deploy has no feature-schema check (local mode allows other schemas by design; needs a decision).</t>
+          <t>2026-10-20 07:13 TC-14 Pass: the raw UNSW-NB15 training file gives exactly the 15 flow features. 10:17 TC-14 Pass on 213d0be: id and attack_cat are dropped from any training file, and train.py warns before training and before --deploy when a model cannot run on captured traffic (Lead Architect decision: warn, not refuse).</t>
         </is>
       </c>
     </row>
@@ -6374,17 +6774,17 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>edf6193 (negative values only)</t>
+          <t>edf6193, 063f42f</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:02 TC-05 re-run: negative values refused at the browser, the form and /predict, nothing stored - Pass for that part. Still open: missing or empty numeric fields are filled with training defaults and stored at the server (deliberate, tested design; needs a decision by the Lead Architect and Product Owner).</t>
+          <t>2026-10-20 07:02: negative values refused, nothing stored. 10:20 TC-05 Pass on 213d0be (Lead Architect decision: refuse missing fields): omitted, null and empty fields refused at the form and /predict with 'Enter a value for every field; missing: dur.', nothing stored.</t>
         </is>
       </c>
     </row>
@@ -6685,7 +7085,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -6695,7 +7095,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:02 USE-01.3 on 0480899: feed, alert, log and report times now say UTC, but Dashboard 'Last at', Nodes, Accounts and local 'Deployed at' did not - fixed in 128855e, whose automated tests passed (07:09). UI re-test on 128855e not executed (app not restarted); stays open until then.</t>
+          <t>2026-10-20 07:02 on 0480899: partly fixed (Dashboard 'Last at', Nodes, Accounts and local 'Deployed at' still unlabelled; fixed in 128855e). 10:20 USE-01.3 Pass on the final build 213d0be: every shown time says UTC.</t>
         </is>
       </c>
     </row>
@@ -7567,7 +7967,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>69% of executed test cases (9 of 13: TC-01, TC-02, TC-04, TC-08, TC-09, TC-10, TC-12, TC-13, TC-16 passed; TC-03, TC-05, TC-11 and TC-14 failed - TC-14 because the DEF-12 re-test still fails; TC-06, TC-07, TC-15 not executed). 76.7% of executed Test Log rows (66 Pass of 86).</t>
+          <t>84.6% of executed test cases (11 of 13: TC-01, TC-02, TC-04, TC-05, TC-08, TC-09, TC-10, TC-12, TC-13, TC-14, TC-16 passed on their latest run; TC-03 and TC-11 failed; TC-06, TC-07, TC-15 not executed). 78.7% of executed Test Log rows (74 Pass of 94, earlier failed runs included).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -7783,7 +8183,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>6 Low/Medium defects open (DEF-08, 10, 11, 12, 16, 17); DEF-01, 02, 03, 09, 13, 14, 15 and 18 fixed and closed in REG-01. DEF-08 and DEF-12 are fixed in part and wait for a decision; DEF-16 waits for its UI re-test on 128855e. Workaround written in DEF-08 (train on 15-feature CSVs); no Product Owner sign-off yet</t>
+          <t>3 Medium defects open (DEF-10, 11, 17 - throughput and lag limits, for cycle 2), without written workarounds; 11 Low/Medium defects (DEF-01, 02, 03, 08, 09, 12, 13, 14, 15, 16, 18) fixed, re-tested and closed. No Product Owner sign-off yet</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -8113,10 +8513,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>5</v>
@@ -8140,10 +8540,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>3</v>
@@ -8194,10 +8594,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>9</v>
@@ -8221,10 +8621,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
test: record the UAT dry run and mark the cycle 2 defects as deferred
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.0.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Owner" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$112</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
@@ -40,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -109,6 +114,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -479,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5774,8 +5782,248 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:43</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01.1</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>UAT scenario 1: replay (Sample traffic 5,000 flows, Fast, Sequential, Save attacks) for about 2 minutes - flows marked Attack/Normal with confidence, Attacks and Alerts Queued rising together, Pending back to 0 and Synced = Queued after Stop, no error.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Dry run on the final build, analyst account, 10:41:35-10:43:35: 169 flows, 123 Attack / 46 Normal, 123 alerts queued, 123 synced, 0 pending, 0 not stored; 50 Recent Flows rows with a verdict on screen; no error message.</t>
+        </is>
+      </c>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/uat/uat_ui.json (scenario1), uat_s1_replay.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:44</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01.2</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>UAT scenario 2: acknowledge then resolve an Open alert - status Acknowledged, then Resolved with a Reopen button; each action once; a Logs entry for each.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Alert #4633 (Open): Acknowledge -&gt; 'Alert #4633 marked Acknowledged.', status Acknowledged; Resolve -&gt; 'Alert #4633 marked Resolved.', status Resolved, Reopen shown and Resolve gone; Logs #5671 'Alert 4633 marked Acknowledged.' and #5672 'Alert 4633 marked Resolved.', one entry each. Rapid double-clicking was not tried.</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/uat/uat_ui.json (scenario2), uat_s2_alerts.png, uat_s2_logs.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:44</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01.3</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>UAT scenario 3: report from three selected alerts - at the top of Operational Reports with type, time (UTC), owner and installation; '3 alerts of evidence' listing the picked alerts; a JSON download.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Alerts #4633, #4632, #4631 selected -&gt; 'Report saved together with its alert evidence.'; Reports top row '#1 Operational evidence 2026-10-20 02:44:08 celpca d535e2fd'; report page 'generated 2026-10-20 02:44:08 UTC - 3 alerts of evidence' listing exactly #4631-#4633; JSON button returns HTTP 200 application/json naming all three alerts.</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>test-results/ui_20261020/uat/uat_ui.json (scenario3), uat_s3_reports.png, uat_s3_report_detail.png; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:44</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01.4</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>UAT scenario 4: an administrator approves a test analyst awaiting approval; the analyst can then monitor without restarting.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Not executed: needs the Administrator account and a test analyst prepared to be awaiting approval on an installation; neither was prepared (passwords are not typed by the test agent, and no accounts are created on the shared pilot for this). The approval flow is covered by the automated test test_enrollment_on_login_and_administrator_approval (tests/test_cloud_app.py) and the Stage 5F pilot.</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Not executed</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>docs/testing/cycle-1/UAT scenarios.md; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 10:44</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>TC-15</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Pauleen Joy O. Gomez</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>213d0be</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner, signed in as an analyst, replays algoguard_big.csv, opens an alert, acknowledges and resolves it: alerts raised for attacks; review actions logged; Product Owner accepts.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>The replay, alert review and report steps were run as a dry run on the final build: alerts raised for attacks (123), review actions logged (UAT-01.1 to UAT-01.3, all Pass); scenario 4 not run. Blocked on the last step: the Product Owner's accept/reject decision and signature on the UAT sheet, to be added later. (Her permission to accept was relayed by the Lead Architect on 2026-10-20; not signed.)</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Test Log rows UAT-01.1 to UAT-01.4; test-results/ui_20261020/uat/; docs/testing/cycle-1/UAT scenarios.md; evidence: product code = 940e082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J107"/>
+  <autoFilter ref="A1:J112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6190,7 +6438,11 @@
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -6262,7 +6514,11 @@
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6334,7 +6590,11 @@
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -6406,7 +6666,11 @@
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -6636,7 +6900,11 @@
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6707,7 +6975,11 @@
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -7168,7 +7440,11 @@
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to test cycle 2 by the Lead Architect (2026-10-20); not fixed or re-tested in cycle 1.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7967,7 +8243,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>84.6% of executed test cases (11 of 13: TC-01, TC-02, TC-04, TC-05, TC-08, TC-09, TC-10, TC-12, TC-13, TC-14, TC-16 passed on their latest run; TC-03 and TC-11 failed; TC-06, TC-07, TC-15 not executed). 78.7% of executed Test Log rows (74 Pass of 94, earlier failed runs included).</t>
+          <t>84.6% of executed test cases (11 of 13: TC-01, TC-02, TC-04, TC-05, TC-08, TC-09, TC-10, TC-12, TC-13, TC-14, TC-16 passed on their latest run; TC-03 and TC-11 failed; TC-06 and TC-07 not executed; TC-15 blocked on the Product Owner's decision). 79.4% of executed Test Log rows (77 Pass of 97, earlier failed runs included).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -8648,23 +8924,23 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Counts are Test Log rows (one per execution, re-runs included). Cases executed = Pass + Fail. Blocked rows are counted under Not executed. Defects are counted against the owner of the card that found them.</t>
         </is>

</xml_diff>